<commit_message>
Antet compact pe „Lista de prețuri”
Antetul înghețat ocupa ~200 px în Google Sheets. Acum: titlu, subtitlu și
rândul cu cursul (tot în F3) + capul de tabel, ~120 px; datele firmei s-au
mutat în notele de la final. Shaktiman și Tractoare regenerate.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XX5MRnGHcF52iH3Y1dYFBw
</commit_message>
<xml_diff>
--- a/output/Lista de preturi - Tractoare.xlsx
+++ b/output/Lista de preturi - Tractoare.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="Curs">'Lista de prețuri'!$F$3</definedName>
     <definedName name="CotaTVA">'Ofertă comercială'!$F$9</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Lista de prețuri'!$6:$6</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Lista de prețuri'!$4:$4</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Ofertă comercială'!$A$1:$H$50</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,13 +24,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="DD.MM.YYYY"/>
-    <numFmt numFmtId="166" formatCode="#,##0 &quot;€&quot;"/>
-    <numFmt numFmtId="167" formatCode="#,##0 &quot;lei&quot;"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="#,##0 &quot;€&quot;"/>
+    <numFmt numFmtId="165" formatCode="#,##0 &quot;lei&quot;"/>
+    <numFmt numFmtId="166" formatCode="DD.MM.YYYY"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="22">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,12 +41,12 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="0000497E"/>
-      <sz val="20"/>
+      <sz val="18"/>
     </font>
     <font>
       <name val="Arial"/>
       <color rgb="00595959"/>
-      <sz val="12"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -62,12 +61,8 @@
     </font>
     <font>
       <name val="Arial"/>
+      <color rgb="00595959"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="00595959"/>
-      <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -83,17 +78,21 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00595959"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00595959"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -123,6 +122,12 @@
       <b val="1"/>
       <color rgb="0000497E"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="0000497E"/>
+      <sz val="20"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -221,7 +226,7 @@
   <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -235,39 +240,38 @@
     <xf numFmtId="2" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="166" fontId="11" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="13" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -277,85 +281,86 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="18" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="19" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="18" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="19" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="17" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="18" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="17" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="18" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -451,9 +456,9 @@
       <col>0</col>
       <colOff>76200</colOff>
       <row>0</row>
-      <rowOff>95250</rowOff>
+      <rowOff>152400</rowOff>
     </from>
-    <ext cx="1428750" cy="495300"/>
+    <ext cx="1266825" cy="438150"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -475,7 +480,7 @@
     <from>
       <col>7</col>
       <colOff>695325</colOff>
-      <row>6</row>
+      <row>4</row>
       <rowOff>57150</rowOff>
     </from>
     <ext cx="1238250" cy="266700"/>
@@ -500,7 +505,7 @@
     <from>
       <col>1</col>
       <colOff>400050</colOff>
-      <row>7</row>
+      <row>5</row>
       <rowOff>28575</rowOff>
     </from>
     <ext cx="514350" cy="514350"/>
@@ -525,7 +530,7 @@
     <from>
       <col>1</col>
       <colOff>419100</colOff>
-      <row>8</row>
+      <row>6</row>
       <rowOff>28575</rowOff>
     </from>
     <ext cx="476250" cy="514350"/>
@@ -550,7 +555,7 @@
     <from>
       <col>1</col>
       <colOff>400050</colOff>
-      <row>9</row>
+      <row>7</row>
       <rowOff>28575</rowOff>
     </from>
     <ext cx="514350" cy="514350"/>
@@ -575,7 +580,7 @@
     <from>
       <col>1</col>
       <colOff>409575</colOff>
-      <row>10</row>
+      <row>8</row>
       <rowOff>28575</rowOff>
     </from>
     <ext cx="485775" cy="514350"/>
@@ -600,7 +605,7 @@
     <from>
       <col>1</col>
       <colOff>390525</colOff>
-      <row>11</row>
+      <row>9</row>
       <rowOff>28575</rowOff>
     </from>
     <ext cx="523875" cy="514350"/>
@@ -625,7 +630,7 @@
     <from>
       <col>1</col>
       <colOff>323850</colOff>
-      <row>12</row>
+      <row>10</row>
       <rowOff>28575</rowOff>
     </from>
     <ext cx="657225" cy="514350"/>
@@ -650,7 +655,7 @@
     <from>
       <col>1</col>
       <colOff>419100</colOff>
-      <row>13</row>
+      <row>11</row>
       <rowOff>28575</rowOff>
     </from>
     <ext cx="476250" cy="514350"/>
@@ -675,7 +680,7 @@
     <from>
       <col>1</col>
       <colOff>409575</colOff>
-      <row>14</row>
+      <row>12</row>
       <rowOff>28575</rowOff>
     </from>
     <ext cx="495300" cy="514350"/>
@@ -700,7 +705,7 @@
     <from>
       <col>1</col>
       <colOff>361950</colOff>
-      <row>15</row>
+      <row>13</row>
       <rowOff>28575</rowOff>
     </from>
     <ext cx="581025" cy="514350"/>
@@ -725,7 +730,7 @@
     <from>
       <col>1</col>
       <colOff>381000</colOff>
-      <row>16</row>
+      <row>14</row>
       <rowOff>28575</rowOff>
     </from>
     <ext cx="542925" cy="514350"/>
@@ -750,7 +755,7 @@
     <from>
       <col>1</col>
       <colOff>419100</colOff>
-      <row>17</row>
+      <row>15</row>
       <rowOff>28575</rowOff>
     </from>
     <ext cx="466725" cy="514350"/>
@@ -775,7 +780,7 @@
     <from>
       <col>1</col>
       <colOff>342900</colOff>
-      <row>18</row>
+      <row>16</row>
       <rowOff>28575</rowOff>
     </from>
     <ext cx="628650" cy="514350"/>
@@ -800,7 +805,7 @@
     <from>
       <col>1</col>
       <colOff>381000</colOff>
-      <row>19</row>
+      <row>17</row>
       <rowOff>28575</rowOff>
     </from>
     <ext cx="542925" cy="514350"/>
@@ -825,7 +830,7 @@
     <from>
       <col>1</col>
       <colOff>361950</colOff>
-      <row>20</row>
+      <row>18</row>
       <rowOff>28575</rowOff>
     </from>
     <ext cx="590550" cy="514350"/>
@@ -850,7 +855,7 @@
     <from>
       <col>7</col>
       <colOff>704850</colOff>
-      <row>21</row>
+      <row>19</row>
       <rowOff>47625</rowOff>
     </from>
     <ext cx="1228725" cy="285750"/>
@@ -875,7 +880,7 @@
     <from>
       <col>1</col>
       <colOff>371475</colOff>
-      <row>22</row>
+      <row>20</row>
       <rowOff>28575</rowOff>
     </from>
     <ext cx="561975" cy="514350"/>
@@ -900,7 +905,7 @@
     <from>
       <col>1</col>
       <colOff>371475</colOff>
-      <row>23</row>
+      <row>21</row>
       <rowOff>28575</rowOff>
     </from>
     <ext cx="571500" cy="514350"/>
@@ -925,7 +930,7 @@
     <from>
       <col>1</col>
       <colOff>400050</colOff>
-      <row>24</row>
+      <row>22</row>
       <rowOff>28575</rowOff>
     </from>
     <ext cx="514350" cy="514350"/>
@@ -950,7 +955,7 @@
     <from>
       <col>1</col>
       <colOff>342900</colOff>
-      <row>25</row>
+      <row>23</row>
       <rowOff>28575</rowOff>
     </from>
     <ext cx="628650" cy="514350"/>
@@ -975,7 +980,7 @@
     <from>
       <col>1</col>
       <colOff>323850</colOff>
-      <row>26</row>
+      <row>24</row>
       <rowOff>28575</rowOff>
     </from>
     <ext cx="657225" cy="514350"/>
@@ -1000,7 +1005,7 @@
     <from>
       <col>1</col>
       <colOff>323850</colOff>
-      <row>27</row>
+      <row>25</row>
       <rowOff>28575</rowOff>
     </from>
     <ext cx="657225" cy="514350"/>
@@ -1025,7 +1030,7 @@
     <from>
       <col>1</col>
       <colOff>381000</colOff>
-      <row>28</row>
+      <row>26</row>
       <rowOff>28575</rowOff>
     </from>
     <ext cx="552450" cy="514350"/>
@@ -1050,7 +1055,7 @@
     <from>
       <col>1</col>
       <colOff>409575</colOff>
-      <row>29</row>
+      <row>27</row>
       <rowOff>28575</rowOff>
     </from>
     <ext cx="485775" cy="514350"/>
@@ -1075,7 +1080,7 @@
     <from>
       <col>7</col>
       <colOff>942975</colOff>
-      <row>30</row>
+      <row>28</row>
       <rowOff>47625</rowOff>
     </from>
     <ext cx="990600" cy="285750"/>
@@ -1100,7 +1105,7 @@
     <from>
       <col>1</col>
       <colOff>314325</colOff>
-      <row>31</row>
+      <row>29</row>
       <rowOff>28575</rowOff>
     </from>
     <ext cx="685800" cy="514350"/>
@@ -1125,7 +1130,7 @@
     <from>
       <col>1</col>
       <colOff>266700</colOff>
-      <row>32</row>
+      <row>30</row>
       <rowOff>28575</rowOff>
     </from>
     <ext cx="771525" cy="514350"/>
@@ -1150,7 +1155,7 @@
     <from>
       <col>1</col>
       <colOff>295275</colOff>
-      <row>33</row>
+      <row>31</row>
       <rowOff>28575</rowOff>
     </from>
     <ext cx="714375" cy="514350"/>
@@ -1175,7 +1180,7 @@
     <from>
       <col>7</col>
       <colOff>1276350</colOff>
-      <row>34</row>
+      <row>32</row>
       <rowOff>47625</rowOff>
     </from>
     <ext cx="657225" cy="285750"/>
@@ -1200,7 +1205,7 @@
     <from>
       <col>1</col>
       <colOff>352425</colOff>
-      <row>35</row>
+      <row>33</row>
       <rowOff>28575</rowOff>
     </from>
     <ext cx="600075" cy="514350"/>
@@ -1225,7 +1230,7 @@
     <from>
       <col>1</col>
       <colOff>342900</colOff>
-      <row>36</row>
+      <row>34</row>
       <rowOff>28575</rowOff>
     </from>
     <ext cx="628650" cy="514350"/>
@@ -1250,7 +1255,7 @@
     <from>
       <col>1</col>
       <colOff>333375</colOff>
-      <row>37</row>
+      <row>35</row>
       <rowOff>28575</rowOff>
     </from>
     <ext cx="647700" cy="514350"/>
@@ -1275,7 +1280,7 @@
     <from>
       <col>1</col>
       <colOff>371475</colOff>
-      <row>38</row>
+      <row>36</row>
       <rowOff>28575</rowOff>
     </from>
     <ext cx="561975" cy="514350"/>
@@ -1300,7 +1305,7 @@
     <from>
       <col>1</col>
       <colOff>381000</colOff>
-      <row>39</row>
+      <row>37</row>
       <rowOff>28575</rowOff>
     </from>
     <ext cx="552450" cy="514350"/>
@@ -1325,7 +1330,7 @@
     <from>
       <col>1</col>
       <colOff>333375</colOff>
-      <row>40</row>
+      <row>38</row>
       <rowOff>28575</rowOff>
     </from>
     <ext cx="647700" cy="514350"/>
@@ -1350,7 +1355,7 @@
     <from>
       <col>1</col>
       <colOff>390525</colOff>
-      <row>41</row>
+      <row>39</row>
       <rowOff>28575</rowOff>
     </from>
     <ext cx="523875" cy="514350"/>
@@ -1375,7 +1380,7 @@
     <from>
       <col>1</col>
       <colOff>323850</colOff>
-      <row>42</row>
+      <row>40</row>
       <rowOff>28575</rowOff>
     </from>
     <ext cx="657225" cy="514350"/>
@@ -1743,7 +1748,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:I46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1757,21 +1762,21 @@
     <col width="16" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="54" customHeight="1">
+    <row r="1" ht="28" customHeight="1">
       <c r="C1" s="1" t="inlineStr">
         <is>
           <t>LISTA DE PREȚURI</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="20" customHeight="1">
+    <row r="2" ht="16" customHeight="1">
       <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Tractoare LS, Farmtrac, Antonio Carraro și Solis</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="22" customHeight="1">
+    <row r="3" ht="20" customHeight="1">
       <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Prețuri în EUR, fără TVA</t>
@@ -1785,1216 +1790,1212 @@
       <c r="F3" s="5" t="n">
         <v>20.1</v>
       </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>Actualizat:</t>
-        </is>
-      </c>
-      <c r="H3" s="6" t="n">
-        <v>46308</v>
-      </c>
-    </row>
-    <row r="4" ht="16" customHeight="1">
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>„Ozonteh Impex” SRL · MD-3701, mun. Strășeni, șos. Chișinău 69, Republica Moldova · office@ozonteh.md · ozonteh.net</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="6" customHeight="1"/>
-    <row r="6" ht="32" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>Actualizat: 13.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>Nr.</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>Foto</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
-        <is>
-          <t>Denumire produs</t>
-        </is>
-      </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Denumire produs</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>Preț EUR
 (fără TVA)</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>Preț promo
 EUR</t>
         </is>
       </c>
-      <c r="F6" s="8" t="inlineStr">
+      <c r="F4" s="7" t="inlineStr">
         <is>
           <t>Preț MDL*
 (fără TVA)</t>
         </is>
       </c>
-      <c r="G6" s="8" t="inlineStr">
+      <c r="G4" s="7" t="inlineStr">
         <is>
           <t>Notă</t>
         </is>
       </c>
-      <c r="H6" s="8" t="inlineStr">
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>Pagina
 produsului</t>
         </is>
       </c>
-      <c r="I6" s="8" t="inlineStr">
+      <c r="I4" s="7" t="inlineStr">
         <is>
           <t>Ofertă
 comercială</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="10" t="inlineStr">
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">  TRACTOARE LS  ·  14 modele</t>
         </is>
       </c>
     </row>
+    <row r="6" ht="46" customHeight="1">
+      <c r="A6" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="11" t="n"/>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>Tractor LS MT1.25 HST FR STAGE V</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="n">
+        <v>12500</v>
+      </c>
+      <c r="E6" s="11" t="n"/>
+      <c r="F6" s="14">
+        <f>IF(ISNUMBER(E6),ROUND(E6*Curs,0),IF(ISNUMBER(D6),ROUND(D6*Curs,0),"La cerere"))</f>
+        <v/>
+      </c>
+      <c r="G6" s="15" t="n"/>
+      <c r="H6" s="16" t="inlineStr">
+        <is>
+          <t>Vezi pe site</t>
+        </is>
+      </c>
+      <c r="I6" s="16" t="inlineStr">
+        <is>
+          <t>Deschide oferta</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="46" customHeight="1">
+      <c r="A7" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" s="11" t="n"/>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>Tractor LS XJ25 MT FR STAGE V</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="n">
+        <v>12500</v>
+      </c>
+      <c r="E7" s="11" t="n"/>
+      <c r="F7" s="14">
+        <f>IF(ISNUMBER(E7),ROUND(E7*Curs,0),IF(ISNUMBER(D7),ROUND(D7*Curs,0),"La cerere"))</f>
+        <v/>
+      </c>
+      <c r="G7" s="15" t="n"/>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>Vezi pe site</t>
+        </is>
+      </c>
+      <c r="I7" s="16" t="inlineStr">
+        <is>
+          <t>Deschide oferta</t>
+        </is>
+      </c>
+    </row>
     <row r="8" ht="46" customHeight="1">
-      <c r="A8" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="B8" s="12" t="n"/>
-      <c r="C8" s="13" t="inlineStr">
-        <is>
-          <t>Tractor LS MT1.25 HST FR STAGE V</t>
-        </is>
-      </c>
-      <c r="D8" s="14" t="n">
-        <v>12500</v>
-      </c>
-      <c r="E8" s="12" t="n"/>
-      <c r="F8" s="15">
+      <c r="A8" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" s="11" t="n"/>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>Tractor LS MT3.40 MT CAB STAGE V</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="n">
+        <v>25000</v>
+      </c>
+      <c r="E8" s="11" t="n"/>
+      <c r="F8" s="14">
         <f>IF(ISNUMBER(E8),ROUND(E8*Curs,0),IF(ISNUMBER(D8),ROUND(D8*Curs,0),"La cerere"))</f>
         <v/>
       </c>
-      <c r="G8" s="16" t="n"/>
-      <c r="H8" s="17" t="inlineStr">
+      <c r="G8" s="15" t="n"/>
+      <c r="H8" s="16" t="inlineStr">
         <is>
           <t>Vezi pe site</t>
         </is>
       </c>
-      <c r="I8" s="17" t="inlineStr">
+      <c r="I8" s="16" t="inlineStr">
         <is>
           <t>Deschide oferta</t>
         </is>
       </c>
     </row>
     <row r="9" ht="46" customHeight="1">
-      <c r="A9" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="B9" s="12" t="n"/>
-      <c r="C9" s="13" t="inlineStr">
-        <is>
-          <t>Tractor LS XJ25 MT FR STAGE V</t>
-        </is>
-      </c>
-      <c r="D9" s="14" t="n">
-        <v>12500</v>
-      </c>
-      <c r="E9" s="12" t="n"/>
-      <c r="F9" s="15">
+      <c r="A9" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" s="11" t="n"/>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>Tractor LS MT3.50 MT CAB STAGE V</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="n">
+        <v>28000</v>
+      </c>
+      <c r="E9" s="11" t="n"/>
+      <c r="F9" s="14">
         <f>IF(ISNUMBER(E9),ROUND(E9*Curs,0),IF(ISNUMBER(D9),ROUND(D9*Curs,0),"La cerere"))</f>
         <v/>
       </c>
-      <c r="G9" s="16" t="n"/>
-      <c r="H9" s="17" t="inlineStr">
+      <c r="G9" s="15" t="n"/>
+      <c r="H9" s="16" t="inlineStr">
         <is>
           <t>Vezi pe site</t>
         </is>
       </c>
-      <c r="I9" s="17" t="inlineStr">
+      <c r="I9" s="16" t="inlineStr">
         <is>
           <t>Deschide oferta</t>
         </is>
       </c>
     </row>
     <row r="10" ht="46" customHeight="1">
-      <c r="A10" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="B10" s="12" t="n"/>
-      <c r="C10" s="13" t="inlineStr">
-        <is>
-          <t>Tractor LS MT3.40 MT CAB STAGE V</t>
-        </is>
-      </c>
-      <c r="D10" s="14" t="n">
+      <c r="A10" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" s="11" t="n"/>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>Tractor LS MT3.60 MT CAB STAGE V</t>
+        </is>
+      </c>
+      <c r="D10" s="13" t="n">
+        <v>30000</v>
+      </c>
+      <c r="E10" s="11" t="n"/>
+      <c r="F10" s="14">
+        <f>IF(ISNUMBER(E10),ROUND(E10*Curs,0),IF(ISNUMBER(D10),ROUND(D10*Curs,0),"La cerere"))</f>
+        <v/>
+      </c>
+      <c r="G10" s="15" t="n"/>
+      <c r="H10" s="16" t="inlineStr">
+        <is>
+          <t>Vezi pe site</t>
+        </is>
+      </c>
+      <c r="I10" s="16" t="inlineStr">
+        <is>
+          <t>Deschide oferta</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="46" customHeight="1">
+      <c r="A11" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="B11" s="11" t="n"/>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>Tractor LS R36i MT FR NON EU</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="n">
+        <v>16500</v>
+      </c>
+      <c r="E11" s="11" t="n"/>
+      <c r="F11" s="14">
+        <f>IF(ISNUMBER(E11),ROUND(E11*Curs,0),IF(ISNUMBER(D11),ROUND(D11*Curs,0),"La cerere"))</f>
+        <v/>
+      </c>
+      <c r="G11" s="15" t="n"/>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>Vezi pe site</t>
+        </is>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>Deschide oferta</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="46" customHeight="1">
+      <c r="A12" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="B12" s="11" t="n"/>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>Tractor LS R60 MT FR NON EU</t>
+        </is>
+      </c>
+      <c r="D12" s="13" t="n">
+        <v>21000</v>
+      </c>
+      <c r="E12" s="17" t="n">
+        <v>19500</v>
+      </c>
+      <c r="F12" s="14">
+        <f>IF(ISNUMBER(E12),ROUND(E12*Curs,0),IF(ISNUMBER(D12),ROUND(D12*Curs,0),"La cerere"))</f>
+        <v/>
+      </c>
+      <c r="G12" s="15" t="n"/>
+      <c r="H12" s="16" t="inlineStr">
+        <is>
+          <t>Vezi pe site</t>
+        </is>
+      </c>
+      <c r="I12" s="16" t="inlineStr">
+        <is>
+          <t>Deschide oferta</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="46" customHeight="1">
+      <c r="A13" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B13" s="11" t="n"/>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>Tractor LS R65 MT CAB NON EU</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="n">
+        <v>29000</v>
+      </c>
+      <c r="E13" s="17" t="n">
+        <v>27500</v>
+      </c>
+      <c r="F13" s="14">
+        <f>IF(ISNUMBER(E13),ROUND(E13*Curs,0),IF(ISNUMBER(D13),ROUND(D13*Curs,0),"La cerere"))</f>
+        <v/>
+      </c>
+      <c r="G13" s="15" t="n"/>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>Vezi pe site</t>
+        </is>
+      </c>
+      <c r="I13" s="16" t="inlineStr">
+        <is>
+          <t>Deschide oferta</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="46" customHeight="1">
+      <c r="A14" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B14" s="11" t="n"/>
+      <c r="C14" s="12" t="inlineStr">
+        <is>
+          <t>Tractor LS XR50 MT CAB NON EU</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="n">
+        <v>26000</v>
+      </c>
+      <c r="E14" s="17" t="n">
         <v>25000</v>
       </c>
-      <c r="E10" s="12" t="n"/>
-      <c r="F10" s="15">
-        <f>IF(ISNUMBER(E10),ROUND(E10*Curs,0),IF(ISNUMBER(D10),ROUND(D10*Curs,0),"La cerere"))</f>
-        <v/>
-      </c>
-      <c r="G10" s="16" t="n"/>
-      <c r="H10" s="17" t="inlineStr">
+      <c r="F14" s="14">
+        <f>IF(ISNUMBER(E14),ROUND(E14*Curs,0),IF(ISNUMBER(D14),ROUND(D14*Curs,0),"La cerere"))</f>
+        <v/>
+      </c>
+      <c r="G14" s="15" t="n"/>
+      <c r="H14" s="16" t="inlineStr">
         <is>
           <t>Vezi pe site</t>
         </is>
       </c>
-      <c r="I10" s="17" t="inlineStr">
+      <c r="I14" s="16" t="inlineStr">
         <is>
           <t>Deschide oferta</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="46" customHeight="1">
-      <c r="A11" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="B11" s="12" t="n"/>
-      <c r="C11" s="13" t="inlineStr">
-        <is>
-          <t>Tractor LS MT3.50 MT CAB STAGE V</t>
-        </is>
-      </c>
-      <c r="D11" s="14" t="n">
+    <row r="15" ht="46" customHeight="1">
+      <c r="A15" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="B15" s="11" t="n"/>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>Tractor LS U60 MT CAB NON EU</t>
+        </is>
+      </c>
+      <c r="D15" s="13" t="n">
+        <v>29500</v>
+      </c>
+      <c r="E15" s="17" t="n">
         <v>28000</v>
       </c>
-      <c r="E11" s="12" t="n"/>
-      <c r="F11" s="15">
-        <f>IF(ISNUMBER(E11),ROUND(E11*Curs,0),IF(ISNUMBER(D11),ROUND(D11*Curs,0),"La cerere"))</f>
-        <v/>
-      </c>
-      <c r="G11" s="16" t="n"/>
-      <c r="H11" s="17" t="inlineStr">
+      <c r="F15" s="14">
+        <f>IF(ISNUMBER(E15),ROUND(E15*Curs,0),IF(ISNUMBER(D15),ROUND(D15*Curs,0),"La cerere"))</f>
+        <v/>
+      </c>
+      <c r="G15" s="15" t="n"/>
+      <c r="H15" s="16" t="inlineStr">
         <is>
           <t>Vezi pe site</t>
         </is>
       </c>
-      <c r="I11" s="17" t="inlineStr">
+      <c r="I15" s="16" t="inlineStr">
         <is>
           <t>Deschide oferta</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="46" customHeight="1">
-      <c r="A12" s="11" t="n">
-        <v>5</v>
-      </c>
-      <c r="B12" s="12" t="n"/>
-      <c r="C12" s="13" t="inlineStr">
-        <is>
-          <t>Tractor LS MT3.60 MT CAB STAGE V</t>
-        </is>
-      </c>
-      <c r="D12" s="14" t="n">
-        <v>30000</v>
-      </c>
-      <c r="E12" s="12" t="n"/>
-      <c r="F12" s="15">
-        <f>IF(ISNUMBER(E12),ROUND(E12*Curs,0),IF(ISNUMBER(D12),ROUND(D12*Curs,0),"La cerere"))</f>
-        <v/>
-      </c>
-      <c r="G12" s="16" t="n"/>
-      <c r="H12" s="17" t="inlineStr">
+    <row r="16" ht="46" customHeight="1">
+      <c r="A16" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="B16" s="11" t="n"/>
+      <c r="C16" s="12" t="inlineStr">
+        <is>
+          <t>Tractor LS XU6168 MT CAB STAGE V</t>
+        </is>
+      </c>
+      <c r="D16" s="13" t="n">
+        <v>33000</v>
+      </c>
+      <c r="E16" s="11" t="n"/>
+      <c r="F16" s="14">
+        <f>IF(ISNUMBER(E16),ROUND(E16*Curs,0),IF(ISNUMBER(D16),ROUND(D16*Curs,0),"La cerere"))</f>
+        <v/>
+      </c>
+      <c r="G16" s="15" t="n"/>
+      <c r="H16" s="16" t="inlineStr">
         <is>
           <t>Vezi pe site</t>
         </is>
       </c>
-      <c r="I12" s="17" t="inlineStr">
+      <c r="I16" s="16" t="inlineStr">
         <is>
           <t>Deschide oferta</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="46" customHeight="1">
-      <c r="A13" s="11" t="n">
-        <v>6</v>
-      </c>
-      <c r="B13" s="12" t="n"/>
-      <c r="C13" s="13" t="inlineStr">
-        <is>
-          <t>Tractor LS R36i MT FR NON EU</t>
-        </is>
-      </c>
-      <c r="D13" s="14" t="n">
-        <v>16500</v>
-      </c>
-      <c r="E13" s="12" t="n"/>
-      <c r="F13" s="15">
-        <f>IF(ISNUMBER(E13),ROUND(E13*Curs,0),IF(ISNUMBER(D13),ROUND(D13*Curs,0),"La cerere"))</f>
-        <v/>
-      </c>
-      <c r="G13" s="16" t="n"/>
-      <c r="H13" s="17" t="inlineStr">
+    <row r="17" ht="46" customHeight="1">
+      <c r="A17" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="B17" s="11" t="n"/>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>Tractor LS MT5.73 PS CAB STAGE V</t>
+        </is>
+      </c>
+      <c r="D17" s="13" t="n">
+        <v>41000</v>
+      </c>
+      <c r="E17" s="11" t="n"/>
+      <c r="F17" s="14">
+        <f>IF(ISNUMBER(E17),ROUND(E17*Curs,0),IF(ISNUMBER(D17),ROUND(D17*Curs,0),"La cerere"))</f>
+        <v/>
+      </c>
+      <c r="G17" s="15" t="n"/>
+      <c r="H17" s="16" t="inlineStr">
         <is>
           <t>Vezi pe site</t>
         </is>
       </c>
-      <c r="I13" s="17" t="inlineStr">
+      <c r="I17" s="16" t="inlineStr">
         <is>
           <t>Deschide oferta</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="46" customHeight="1">
-      <c r="A14" s="11" t="n">
-        <v>7</v>
-      </c>
-      <c r="B14" s="12" t="n"/>
-      <c r="C14" s="13" t="inlineStr">
-        <is>
-          <t>Tractor LS R60 MT FR NON EU</t>
-        </is>
-      </c>
-      <c r="D14" s="14" t="n">
-        <v>21000</v>
-      </c>
-      <c r="E14" s="18" t="n">
+    <row r="18" ht="46" customHeight="1">
+      <c r="A18" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="B18" s="11" t="n"/>
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>Tractor LS PLUS100 PS CAB NON EU</t>
+        </is>
+      </c>
+      <c r="D18" s="13" t="n">
+        <v>43000</v>
+      </c>
+      <c r="E18" s="17" t="n">
+        <v>41000</v>
+      </c>
+      <c r="F18" s="14">
+        <f>IF(ISNUMBER(E18),ROUND(E18*Curs,0),IF(ISNUMBER(D18),ROUND(D18*Curs,0),"La cerere"))</f>
+        <v/>
+      </c>
+      <c r="G18" s="15" t="n"/>
+      <c r="H18" s="16" t="inlineStr">
+        <is>
+          <t>Vezi pe site</t>
+        </is>
+      </c>
+      <c r="I18" s="16" t="inlineStr">
+        <is>
+          <t>Deschide oferta</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="46" customHeight="1">
+      <c r="A19" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="B19" s="11" t="n"/>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>Tractor LS MT7.101 PS CAB STAGE V</t>
+        </is>
+      </c>
+      <c r="D19" s="13" t="n">
+        <v>53000</v>
+      </c>
+      <c r="E19" s="11" t="n"/>
+      <c r="F19" s="14">
+        <f>IF(ISNUMBER(E19),ROUND(E19*Curs,0),IF(ISNUMBER(D19),ROUND(D19*Curs,0),"La cerere"))</f>
+        <v/>
+      </c>
+      <c r="G19" s="15" t="n"/>
+      <c r="H19" s="16" t="inlineStr">
+        <is>
+          <t>Vezi pe site</t>
+        </is>
+      </c>
+      <c r="I19" s="16" t="inlineStr">
+        <is>
+          <t>Deschide oferta</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  TRACTOARE FARMTRAC  ·  8 modele</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="46" customHeight="1">
+      <c r="A21" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="B21" s="11" t="n"/>
+      <c r="C21" s="12" t="inlineStr">
+        <is>
+          <t>Set tractor Farmtrac 26 + freză Shaktiman</t>
+        </is>
+      </c>
+      <c r="D21" s="13" t="n">
+        <v>9900</v>
+      </c>
+      <c r="E21" s="17" t="n">
+        <v>9000</v>
+      </c>
+      <c r="F21" s="14">
+        <f>IF(ISNUMBER(E21),ROUND(E21*Curs,0),IF(ISNUMBER(D21),ROUND(D21*Curs,0),"La cerere"))</f>
+        <v/>
+      </c>
+      <c r="G21" s="15" t="inlineStr">
+        <is>
+          <t>Ofertă de iarnă</t>
+        </is>
+      </c>
+      <c r="H21" s="16" t="inlineStr">
+        <is>
+          <t>Vezi pe site</t>
+        </is>
+      </c>
+      <c r="I21" s="16" t="inlineStr">
+        <is>
+          <t>Deschide oferta</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="46" customHeight="1">
+      <c r="A22" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="B22" s="11" t="n"/>
+      <c r="C22" s="12" t="inlineStr">
+        <is>
+          <t>Tractor Farmtrac 26 4WD</t>
+        </is>
+      </c>
+      <c r="D22" s="13" t="n">
+        <v>8500</v>
+      </c>
+      <c r="E22" s="17" t="n">
+        <v>8000</v>
+      </c>
+      <c r="F22" s="14">
+        <f>IF(ISNUMBER(E22),ROUND(E22*Curs,0),IF(ISNUMBER(D22),ROUND(D22*Curs,0),"La cerere"))</f>
+        <v/>
+      </c>
+      <c r="G22" s="15" t="n"/>
+      <c r="H22" s="16" t="inlineStr">
+        <is>
+          <t>Vezi pe site</t>
+        </is>
+      </c>
+      <c r="I22" s="16" t="inlineStr">
+        <is>
+          <t>Deschide oferta</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="46" customHeight="1">
+      <c r="A23" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="B23" s="11" t="n"/>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>Tractor Farmtrac 26 Pro 4WD</t>
+        </is>
+      </c>
+      <c r="D23" s="13" t="n">
+        <v>8500</v>
+      </c>
+      <c r="E23" s="11" t="n"/>
+      <c r="F23" s="14">
+        <f>IF(ISNUMBER(E23),ROUND(E23*Curs,0),IF(ISNUMBER(D23),ROUND(D23*Curs,0),"La cerere"))</f>
+        <v/>
+      </c>
+      <c r="G23" s="15" t="inlineStr">
+        <is>
+          <t>Model nou, Stage 5, 9x9</t>
+        </is>
+      </c>
+      <c r="H23" s="16" t="inlineStr">
+        <is>
+          <t>Vezi pe site</t>
+        </is>
+      </c>
+      <c r="I23" s="16" t="inlineStr">
+        <is>
+          <t>Deschide oferta</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="46" customHeight="1">
+      <c r="A24" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="B24" s="11" t="n"/>
+      <c r="C24" s="12" t="inlineStr">
+        <is>
+          <t>Tractor Farmtrac 30 4WD</t>
+        </is>
+      </c>
+      <c r="D24" s="13" t="n">
+        <v>9000</v>
+      </c>
+      <c r="E24" s="11" t="n"/>
+      <c r="F24" s="14">
+        <f>IF(ISNUMBER(E24),ROUND(E24*Curs,0),IF(ISNUMBER(D24),ROUND(D24*Curs,0),"La cerere"))</f>
+        <v/>
+      </c>
+      <c r="G24" s="15" t="n"/>
+      <c r="H24" s="16" t="inlineStr">
+        <is>
+          <t>Vezi pe site</t>
+        </is>
+      </c>
+      <c r="I24" s="16" t="inlineStr">
+        <is>
+          <t>Deschide oferta</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="46" customHeight="1">
+      <c r="A25" s="10" t="n">
+        <v>19</v>
+      </c>
+      <c r="B25" s="11" t="n"/>
+      <c r="C25" s="12" t="inlineStr">
+        <is>
+          <t>Tractor Farmtrac 35 4WD</t>
+        </is>
+      </c>
+      <c r="D25" s="13" t="n">
+        <v>9500</v>
+      </c>
+      <c r="E25" s="11" t="n"/>
+      <c r="F25" s="14">
+        <f>IF(ISNUMBER(E25),ROUND(E25*Curs,0),IF(ISNUMBER(D25),ROUND(D25*Curs,0),"La cerere"))</f>
+        <v/>
+      </c>
+      <c r="G25" s="15" t="n"/>
+      <c r="H25" s="16" t="inlineStr">
+        <is>
+          <t>Vezi pe site</t>
+        </is>
+      </c>
+      <c r="I25" s="16" t="inlineStr">
+        <is>
+          <t>Deschide oferta</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="46" customHeight="1">
+      <c r="A26" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="B26" s="11" t="n"/>
+      <c r="C26" s="12" t="inlineStr">
+        <is>
+          <t>Tractor Farmtrac 35 4WD Revers</t>
+        </is>
+      </c>
+      <c r="D26" s="13" t="n">
+        <v>9800</v>
+      </c>
+      <c r="E26" s="11" t="n"/>
+      <c r="F26" s="14">
+        <f>IF(ISNUMBER(E26),ROUND(E26*Curs,0),IF(ISNUMBER(D26),ROUND(D26*Curs,0),"La cerere"))</f>
+        <v/>
+      </c>
+      <c r="G26" s="15" t="n"/>
+      <c r="H26" s="16" t="inlineStr">
+        <is>
+          <t>Vezi pe site</t>
+        </is>
+      </c>
+      <c r="I26" s="16" t="inlineStr">
+        <is>
+          <t>Deschide oferta</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="46" customHeight="1">
+      <c r="A27" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="B27" s="11" t="n"/>
+      <c r="C27" s="12" t="inlineStr">
+        <is>
+          <t>Tractor Farmtrac 6075N 4WD</t>
+        </is>
+      </c>
+      <c r="D27" s="13" t="n">
         <v>19500</v>
       </c>
-      <c r="F14" s="15">
-        <f>IF(ISNUMBER(E14),ROUND(E14*Curs,0),IF(ISNUMBER(D14),ROUND(D14*Curs,0),"La cerere"))</f>
-        <v/>
-      </c>
-      <c r="G14" s="16" t="n"/>
-      <c r="H14" s="17" t="inlineStr">
+      <c r="E27" s="17" t="n">
+        <v>16999</v>
+      </c>
+      <c r="F27" s="14">
+        <f>IF(ISNUMBER(E27),ROUND(E27*Curs,0),IF(ISNUMBER(D27),ROUND(D27*Curs,0),"La cerere"))</f>
+        <v/>
+      </c>
+      <c r="G27" s="15" t="n"/>
+      <c r="H27" s="16" t="inlineStr">
         <is>
           <t>Vezi pe site</t>
         </is>
       </c>
-      <c r="I14" s="17" t="inlineStr">
+      <c r="I27" s="16" t="inlineStr">
         <is>
           <t>Deschide oferta</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="46" customHeight="1">
-      <c r="A15" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="B15" s="12" t="n"/>
-      <c r="C15" s="13" t="inlineStr">
-        <is>
-          <t>Tractor LS R65 MT CAB NON EU</t>
-        </is>
-      </c>
-      <c r="D15" s="14" t="n">
-        <v>29000</v>
-      </c>
-      <c r="E15" s="18" t="n">
+    <row r="28" ht="46" customHeight="1">
+      <c r="A28" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="B28" s="11" t="n"/>
+      <c r="C28" s="12" t="inlineStr">
+        <is>
+          <t>Tractor Farmtrac 6075N 4WD Cabină</t>
+        </is>
+      </c>
+      <c r="D28" s="13" t="n">
+        <v>24500</v>
+      </c>
+      <c r="E28" s="17" t="n">
+        <v>23000</v>
+      </c>
+      <c r="F28" s="14">
+        <f>IF(ISNUMBER(E28),ROUND(E28*Curs,0),IF(ISNUMBER(D28),ROUND(D28*Curs,0),"La cerere"))</f>
+        <v/>
+      </c>
+      <c r="G28" s="15" t="n"/>
+      <c r="H28" s="16" t="inlineStr">
+        <is>
+          <t>Vezi pe site</t>
+        </is>
+      </c>
+      <c r="I28" s="16" t="inlineStr">
+        <is>
+          <t>Deschide oferta</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  TRACTOARE ANTONIO CARRARO  ·  3 modele</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="46" customHeight="1">
+      <c r="A30" s="10" t="n">
+        <v>23</v>
+      </c>
+      <c r="B30" s="11" t="n"/>
+      <c r="C30" s="12" t="inlineStr">
+        <is>
+          <t>Tractor Antonio Carraro AV2100L</t>
+        </is>
+      </c>
+      <c r="D30" s="13" t="n">
+        <v>48000</v>
+      </c>
+      <c r="E30" s="11" t="n"/>
+      <c r="F30" s="14">
+        <f>IF(ISNUMBER(E30),ROUND(E30*Curs,0),IF(ISNUMBER(D30),ROUND(D30*Curs,0),"La cerere"))</f>
+        <v/>
+      </c>
+      <c r="G30" s="15" t="n"/>
+      <c r="H30" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I30" s="16" t="inlineStr">
+        <is>
+          <t>Deschide oferta</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="46" customHeight="1">
+      <c r="A31" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="B31" s="11" t="n"/>
+      <c r="C31" s="12" t="inlineStr">
+        <is>
+          <t>Tractor Antonio Carraro TGF 9900</t>
+        </is>
+      </c>
+      <c r="D31" s="13" t="n">
+        <v>45000</v>
+      </c>
+      <c r="E31" s="11" t="n"/>
+      <c r="F31" s="14">
+        <f>IF(ISNUMBER(E31),ROUND(E31*Curs,0),IF(ISNUMBER(D31),ROUND(D31*Curs,0),"La cerere"))</f>
+        <v/>
+      </c>
+      <c r="G31" s="15" t="n"/>
+      <c r="H31" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I31" s="16" t="inlineStr">
+        <is>
+          <t>Deschide oferta</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="46" customHeight="1">
+      <c r="A32" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="B32" s="11" t="n"/>
+      <c r="C32" s="12" t="inlineStr">
+        <is>
+          <t>Tractor Antonio Carraro TRG 9900</t>
+        </is>
+      </c>
+      <c r="D32" s="13" t="n">
+        <v>48000</v>
+      </c>
+      <c r="E32" s="11" t="n"/>
+      <c r="F32" s="14">
+        <f>IF(ISNUMBER(E32),ROUND(E32*Curs,0),IF(ISNUMBER(D32),ROUND(D32*Curs,0),"La cerere"))</f>
+        <v/>
+      </c>
+      <c r="G32" s="15" t="inlineStr">
+        <is>
+          <t>Reversibil</t>
+        </is>
+      </c>
+      <c r="H32" s="16" t="inlineStr">
+        <is>
+          <t>Vezi pe site</t>
+        </is>
+      </c>
+      <c r="I32" s="16" t="inlineStr">
+        <is>
+          <t>Deschide oferta</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="30" customHeight="1">
+      <c r="A33" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  TRACTOARE SOLIS  ·  8 modele</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="46" customHeight="1">
+      <c r="A34" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="B34" s="11" t="n"/>
+      <c r="C34" s="12" t="inlineStr">
+        <is>
+          <t>Tractor Solis S16</t>
+        </is>
+      </c>
+      <c r="D34" s="13" t="n">
+        <v>6000</v>
+      </c>
+      <c r="E34" s="11" t="n"/>
+      <c r="F34" s="14">
+        <f>IF(ISNUMBER(E34),ROUND(E34*Curs,0),IF(ISNUMBER(D34),ROUND(D34*Curs,0),"La cerere"))</f>
+        <v/>
+      </c>
+      <c r="G34" s="15" t="n"/>
+      <c r="H34" s="16" t="inlineStr">
+        <is>
+          <t>Vezi pe site</t>
+        </is>
+      </c>
+      <c r="I34" s="16" t="inlineStr">
+        <is>
+          <t>Deschide oferta</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="46" customHeight="1">
+      <c r="A35" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="B35" s="11" t="n"/>
+      <c r="C35" s="12" t="inlineStr">
+        <is>
+          <t>Tractor Solis S26</t>
+        </is>
+      </c>
+      <c r="D35" s="13" t="n">
+        <v>8000</v>
+      </c>
+      <c r="E35" s="11" t="n"/>
+      <c r="F35" s="14">
+        <f>IF(ISNUMBER(E35),ROUND(E35*Curs,0),IF(ISNUMBER(D35),ROUND(D35*Curs,0),"La cerere"))</f>
+        <v/>
+      </c>
+      <c r="G35" s="15" t="n"/>
+      <c r="H35" s="16" t="inlineStr">
+        <is>
+          <t>Vezi pe site</t>
+        </is>
+      </c>
+      <c r="I35" s="16" t="inlineStr">
+        <is>
+          <t>Deschide oferta</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="46" customHeight="1">
+      <c r="A36" s="10" t="n">
+        <v>28</v>
+      </c>
+      <c r="B36" s="11" t="n"/>
+      <c r="C36" s="12" t="inlineStr">
+        <is>
+          <t>Tractor Solis S26 Xtra</t>
+        </is>
+      </c>
+      <c r="D36" s="13" t="n">
+        <v>8300</v>
+      </c>
+      <c r="E36" s="11" t="n"/>
+      <c r="F36" s="14">
+        <f>IF(ISNUMBER(E36),ROUND(E36*Curs,0),IF(ISNUMBER(D36),ROUND(D36*Curs,0),"La cerere"))</f>
+        <v/>
+      </c>
+      <c r="G36" s="15" t="n"/>
+      <c r="H36" s="16" t="inlineStr">
+        <is>
+          <t>Vezi pe site</t>
+        </is>
+      </c>
+      <c r="I36" s="16" t="inlineStr">
+        <is>
+          <t>Deschide oferta</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="46" customHeight="1">
+      <c r="A37" s="10" t="n">
+        <v>29</v>
+      </c>
+      <c r="B37" s="11" t="n"/>
+      <c r="C37" s="12" t="inlineStr">
+        <is>
+          <t>Tractor Solis S26 Shuttle XL</t>
+        </is>
+      </c>
+      <c r="D37" s="13" t="n">
+        <v>8500</v>
+      </c>
+      <c r="E37" s="11" t="n"/>
+      <c r="F37" s="14">
+        <f>IF(ISNUMBER(E37),ROUND(E37*Curs,0),IF(ISNUMBER(D37),ROUND(D37*Curs,0),"La cerere"))</f>
+        <v/>
+      </c>
+      <c r="G37" s="15" t="n"/>
+      <c r="H37" s="16" t="inlineStr">
+        <is>
+          <t>Vezi pe site</t>
+        </is>
+      </c>
+      <c r="I37" s="16" t="inlineStr">
+        <is>
+          <t>Deschide oferta</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="46" customHeight="1">
+      <c r="A38" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="B38" s="11" t="n"/>
+      <c r="C38" s="12" t="inlineStr">
+        <is>
+          <t>Tractor Solis S30</t>
+        </is>
+      </c>
+      <c r="D38" s="13" t="n">
+        <v>8700</v>
+      </c>
+      <c r="E38" s="11" t="n"/>
+      <c r="F38" s="14">
+        <f>IF(ISNUMBER(E38),ROUND(E38*Curs,0),IF(ISNUMBER(D38),ROUND(D38*Curs,0),"La cerere"))</f>
+        <v/>
+      </c>
+      <c r="G38" s="15" t="n"/>
+      <c r="H38" s="16" t="inlineStr">
+        <is>
+          <t>Vezi pe site</t>
+        </is>
+      </c>
+      <c r="I38" s="16" t="inlineStr">
+        <is>
+          <t>Deschide oferta</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="46" customHeight="1">
+      <c r="A39" s="10" t="n">
+        <v>31</v>
+      </c>
+      <c r="B39" s="11" t="n"/>
+      <c r="C39" s="12" t="inlineStr">
+        <is>
+          <t>Tractor Solis S32</t>
+        </is>
+      </c>
+      <c r="D39" s="13" t="n">
+        <v>9100</v>
+      </c>
+      <c r="E39" s="11" t="n"/>
+      <c r="F39" s="14">
+        <f>IF(ISNUMBER(E39),ROUND(E39*Curs,0),IF(ISNUMBER(D39),ROUND(D39*Curs,0),"La cerere"))</f>
+        <v/>
+      </c>
+      <c r="G39" s="15" t="n"/>
+      <c r="H39" s="16" t="inlineStr">
+        <is>
+          <t>Vezi pe site</t>
+        </is>
+      </c>
+      <c r="I39" s="16" t="inlineStr">
+        <is>
+          <t>Deschide oferta</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="46" customHeight="1">
+      <c r="A40" s="10" t="n">
+        <v>32</v>
+      </c>
+      <c r="B40" s="11" t="n"/>
+      <c r="C40" s="12" t="inlineStr">
+        <is>
+          <t>Tractor Solis 90N</t>
+        </is>
+      </c>
+      <c r="D40" s="13" t="n">
+        <v>29500</v>
+      </c>
+      <c r="E40" s="11" t="n"/>
+      <c r="F40" s="14">
+        <f>IF(ISNUMBER(E40),ROUND(E40*Curs,0),IF(ISNUMBER(D40),ROUND(D40*Curs,0),"La cerere"))</f>
+        <v/>
+      </c>
+      <c r="G40" s="15" t="n"/>
+      <c r="H40" s="16" t="inlineStr">
+        <is>
+          <t>Vezi pe site</t>
+        </is>
+      </c>
+      <c r="I40" s="16" t="inlineStr">
+        <is>
+          <t>Deschide oferta</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="46" customHeight="1">
+      <c r="A41" s="10" t="n">
+        <v>33</v>
+      </c>
+      <c r="B41" s="11" t="n"/>
+      <c r="C41" s="12" t="inlineStr">
+        <is>
+          <t>Tractor Solis 90RX</t>
+        </is>
+      </c>
+      <c r="D41" s="13" t="n">
         <v>27500</v>
       </c>
-      <c r="F15" s="15">
-        <f>IF(ISNUMBER(E15),ROUND(E15*Curs,0),IF(ISNUMBER(D15),ROUND(D15*Curs,0),"La cerere"))</f>
-        <v/>
-      </c>
-      <c r="G15" s="16" t="n"/>
-      <c r="H15" s="17" t="inlineStr">
+      <c r="E41" s="11" t="n"/>
+      <c r="F41" s="14">
+        <f>IF(ISNUMBER(E41),ROUND(E41*Curs,0),IF(ISNUMBER(D41),ROUND(D41*Curs,0),"La cerere"))</f>
+        <v/>
+      </c>
+      <c r="G41" s="15" t="n"/>
+      <c r="H41" s="16" t="inlineStr">
         <is>
           <t>Vezi pe site</t>
         </is>
       </c>
-      <c r="I15" s="17" t="inlineStr">
+      <c r="I41" s="16" t="inlineStr">
         <is>
           <t>Deschide oferta</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="46" customHeight="1">
-      <c r="A16" s="11" t="n">
-        <v>9</v>
-      </c>
-      <c r="B16" s="12" t="n"/>
-      <c r="C16" s="13" t="inlineStr">
-        <is>
-          <t>Tractor LS XR50 MT CAB NON EU</t>
-        </is>
-      </c>
-      <c r="D16" s="14" t="n">
-        <v>26000</v>
-      </c>
-      <c r="E16" s="18" t="n">
-        <v>25000</v>
-      </c>
-      <c r="F16" s="15">
-        <f>IF(ISNUMBER(E16),ROUND(E16*Curs,0),IF(ISNUMBER(D16),ROUND(D16*Curs,0),"La cerere"))</f>
-        <v/>
-      </c>
-      <c r="G16" s="16" t="n"/>
-      <c r="H16" s="17" t="inlineStr">
-        <is>
-          <t>Vezi pe site</t>
-        </is>
-      </c>
-      <c r="I16" s="17" t="inlineStr">
-        <is>
-          <t>Deschide oferta</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="46" customHeight="1">
-      <c r="A17" s="11" t="n">
-        <v>10</v>
-      </c>
-      <c r="B17" s="12" t="n"/>
-      <c r="C17" s="13" t="inlineStr">
-        <is>
-          <t>Tractor LS U60 MT CAB NON EU</t>
-        </is>
-      </c>
-      <c r="D17" s="14" t="n">
-        <v>29500</v>
-      </c>
-      <c r="E17" s="18" t="n">
-        <v>28000</v>
-      </c>
-      <c r="F17" s="15">
-        <f>IF(ISNUMBER(E17),ROUND(E17*Curs,0),IF(ISNUMBER(D17),ROUND(D17*Curs,0),"La cerere"))</f>
-        <v/>
-      </c>
-      <c r="G17" s="16" t="n"/>
-      <c r="H17" s="17" t="inlineStr">
-        <is>
-          <t>Vezi pe site</t>
-        </is>
-      </c>
-      <c r="I17" s="17" t="inlineStr">
-        <is>
-          <t>Deschide oferta</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="46" customHeight="1">
-      <c r="A18" s="11" t="n">
-        <v>11</v>
-      </c>
-      <c r="B18" s="12" t="n"/>
-      <c r="C18" s="13" t="inlineStr">
-        <is>
-          <t>Tractor LS XU6168 MT CAB STAGE V</t>
-        </is>
-      </c>
-      <c r="D18" s="14" t="n">
-        <v>33000</v>
-      </c>
-      <c r="E18" s="12" t="n"/>
-      <c r="F18" s="15">
-        <f>IF(ISNUMBER(E18),ROUND(E18*Curs,0),IF(ISNUMBER(D18),ROUND(D18*Curs,0),"La cerere"))</f>
-        <v/>
-      </c>
-      <c r="G18" s="16" t="n"/>
-      <c r="H18" s="17" t="inlineStr">
-        <is>
-          <t>Vezi pe site</t>
-        </is>
-      </c>
-      <c r="I18" s="17" t="inlineStr">
-        <is>
-          <t>Deschide oferta</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="46" customHeight="1">
-      <c r="A19" s="11" t="n">
-        <v>12</v>
-      </c>
-      <c r="B19" s="12" t="n"/>
-      <c r="C19" s="13" t="inlineStr">
-        <is>
-          <t>Tractor LS MT5.73 PS CAB STAGE V</t>
-        </is>
-      </c>
-      <c r="D19" s="14" t="n">
-        <v>41000</v>
-      </c>
-      <c r="E19" s="12" t="n"/>
-      <c r="F19" s="15">
-        <f>IF(ISNUMBER(E19),ROUND(E19*Curs,0),IF(ISNUMBER(D19),ROUND(D19*Curs,0),"La cerere"))</f>
-        <v/>
-      </c>
-      <c r="G19" s="16" t="n"/>
-      <c r="H19" s="17" t="inlineStr">
-        <is>
-          <t>Vezi pe site</t>
-        </is>
-      </c>
-      <c r="I19" s="17" t="inlineStr">
-        <is>
-          <t>Deschide oferta</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="46" customHeight="1">
-      <c r="A20" s="11" t="n">
-        <v>13</v>
-      </c>
-      <c r="B20" s="12" t="n"/>
-      <c r="C20" s="13" t="inlineStr">
-        <is>
-          <t>Tractor LS PLUS100 PS CAB NON EU</t>
-        </is>
-      </c>
-      <c r="D20" s="14" t="n">
-        <v>43000</v>
-      </c>
-      <c r="E20" s="18" t="n">
-        <v>41000</v>
-      </c>
-      <c r="F20" s="15">
-        <f>IF(ISNUMBER(E20),ROUND(E20*Curs,0),IF(ISNUMBER(D20),ROUND(D20*Curs,0),"La cerere"))</f>
-        <v/>
-      </c>
-      <c r="G20" s="16" t="n"/>
-      <c r="H20" s="17" t="inlineStr">
-        <is>
-          <t>Vezi pe site</t>
-        </is>
-      </c>
-      <c r="I20" s="17" t="inlineStr">
-        <is>
-          <t>Deschide oferta</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="46" customHeight="1">
-      <c r="A21" s="11" t="n">
-        <v>14</v>
-      </c>
-      <c r="B21" s="12" t="n"/>
-      <c r="C21" s="13" t="inlineStr">
-        <is>
-          <t>Tractor LS MT7.101 PS CAB STAGE V</t>
-        </is>
-      </c>
-      <c r="D21" s="14" t="n">
-        <v>53000</v>
-      </c>
-      <c r="E21" s="12" t="n"/>
-      <c r="F21" s="15">
-        <f>IF(ISNUMBER(E21),ROUND(E21*Curs,0),IF(ISNUMBER(D21),ROUND(D21*Curs,0),"La cerere"))</f>
-        <v/>
-      </c>
-      <c r="G21" s="16" t="n"/>
-      <c r="H21" s="17" t="inlineStr">
-        <is>
-          <t>Vezi pe site</t>
-        </is>
-      </c>
-      <c r="I21" s="17" t="inlineStr">
-        <is>
-          <t>Deschide oferta</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  TRACTOARE FARMTRAC  ·  8 modele</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="46" customHeight="1">
-      <c r="A23" s="11" t="n">
-        <v>15</v>
-      </c>
-      <c r="B23" s="12" t="n"/>
-      <c r="C23" s="13" t="inlineStr">
-        <is>
-          <t>Set tractor Farmtrac 26 + freză Shaktiman</t>
-        </is>
-      </c>
-      <c r="D23" s="14" t="n">
-        <v>9900</v>
-      </c>
-      <c r="E23" s="18" t="n">
-        <v>9000</v>
-      </c>
-      <c r="F23" s="15">
-        <f>IF(ISNUMBER(E23),ROUND(E23*Curs,0),IF(ISNUMBER(D23),ROUND(D23*Curs,0),"La cerere"))</f>
-        <v/>
-      </c>
-      <c r="G23" s="16" t="inlineStr">
-        <is>
-          <t>Ofertă de iarnă</t>
-        </is>
-      </c>
-      <c r="H23" s="17" t="inlineStr">
-        <is>
-          <t>Vezi pe site</t>
-        </is>
-      </c>
-      <c r="I23" s="17" t="inlineStr">
-        <is>
-          <t>Deschide oferta</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="46" customHeight="1">
-      <c r="A24" s="11" t="n">
-        <v>16</v>
-      </c>
-      <c r="B24" s="12" t="n"/>
-      <c r="C24" s="13" t="inlineStr">
-        <is>
-          <t>Tractor Farmtrac 26 4WD</t>
-        </is>
-      </c>
-      <c r="D24" s="14" t="n">
-        <v>8500</v>
-      </c>
-      <c r="E24" s="18" t="n">
-        <v>8000</v>
-      </c>
-      <c r="F24" s="15">
-        <f>IF(ISNUMBER(E24),ROUND(E24*Curs,0),IF(ISNUMBER(D24),ROUND(D24*Curs,0),"La cerere"))</f>
-        <v/>
-      </c>
-      <c r="G24" s="16" t="n"/>
-      <c r="H24" s="17" t="inlineStr">
-        <is>
-          <t>Vezi pe site</t>
-        </is>
-      </c>
-      <c r="I24" s="17" t="inlineStr">
-        <is>
-          <t>Deschide oferta</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="46" customHeight="1">
-      <c r="A25" s="11" t="n">
-        <v>17</v>
-      </c>
-      <c r="B25" s="12" t="n"/>
-      <c r="C25" s="13" t="inlineStr">
-        <is>
-          <t>Tractor Farmtrac 26 Pro 4WD</t>
-        </is>
-      </c>
-      <c r="D25" s="14" t="n">
-        <v>8500</v>
-      </c>
-      <c r="E25" s="12" t="n"/>
-      <c r="F25" s="15">
-        <f>IF(ISNUMBER(E25),ROUND(E25*Curs,0),IF(ISNUMBER(D25),ROUND(D25*Curs,0),"La cerere"))</f>
-        <v/>
-      </c>
-      <c r="G25" s="16" t="inlineStr">
-        <is>
-          <t>Model nou, Stage 5, 9x9</t>
-        </is>
-      </c>
-      <c r="H25" s="17" t="inlineStr">
-        <is>
-          <t>Vezi pe site</t>
-        </is>
-      </c>
-      <c r="I25" s="17" t="inlineStr">
-        <is>
-          <t>Deschide oferta</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="46" customHeight="1">
-      <c r="A26" s="11" t="n">
-        <v>18</v>
-      </c>
-      <c r="B26" s="12" t="n"/>
-      <c r="C26" s="13" t="inlineStr">
-        <is>
-          <t>Tractor Farmtrac 30 4WD</t>
-        </is>
-      </c>
-      <c r="D26" s="14" t="n">
-        <v>9000</v>
-      </c>
-      <c r="E26" s="12" t="n"/>
-      <c r="F26" s="15">
-        <f>IF(ISNUMBER(E26),ROUND(E26*Curs,0),IF(ISNUMBER(D26),ROUND(D26*Curs,0),"La cerere"))</f>
-        <v/>
-      </c>
-      <c r="G26" s="16" t="n"/>
-      <c r="H26" s="17" t="inlineStr">
-        <is>
-          <t>Vezi pe site</t>
-        </is>
-      </c>
-      <c r="I26" s="17" t="inlineStr">
-        <is>
-          <t>Deschide oferta</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="46" customHeight="1">
-      <c r="A27" s="11" t="n">
-        <v>19</v>
-      </c>
-      <c r="B27" s="12" t="n"/>
-      <c r="C27" s="13" t="inlineStr">
-        <is>
-          <t>Tractor Farmtrac 35 4WD</t>
-        </is>
-      </c>
-      <c r="D27" s="14" t="n">
-        <v>9500</v>
-      </c>
-      <c r="E27" s="12" t="n"/>
-      <c r="F27" s="15">
-        <f>IF(ISNUMBER(E27),ROUND(E27*Curs,0),IF(ISNUMBER(D27),ROUND(D27*Curs,0),"La cerere"))</f>
-        <v/>
-      </c>
-      <c r="G27" s="16" t="n"/>
-      <c r="H27" s="17" t="inlineStr">
-        <is>
-          <t>Vezi pe site</t>
-        </is>
-      </c>
-      <c r="I27" s="17" t="inlineStr">
-        <is>
-          <t>Deschide oferta</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="46" customHeight="1">
-      <c r="A28" s="11" t="n">
-        <v>20</v>
-      </c>
-      <c r="B28" s="12" t="n"/>
-      <c r="C28" s="13" t="inlineStr">
-        <is>
-          <t>Tractor Farmtrac 35 4WD Revers</t>
-        </is>
-      </c>
-      <c r="D28" s="14" t="n">
-        <v>9800</v>
-      </c>
-      <c r="E28" s="12" t="n"/>
-      <c r="F28" s="15">
-        <f>IF(ISNUMBER(E28),ROUND(E28*Curs,0),IF(ISNUMBER(D28),ROUND(D28*Curs,0),"La cerere"))</f>
-        <v/>
-      </c>
-      <c r="G28" s="16" t="n"/>
-      <c r="H28" s="17" t="inlineStr">
-        <is>
-          <t>Vezi pe site</t>
-        </is>
-      </c>
-      <c r="I28" s="17" t="inlineStr">
-        <is>
-          <t>Deschide oferta</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="46" customHeight="1">
-      <c r="A29" s="11" t="n">
-        <v>21</v>
-      </c>
-      <c r="B29" s="12" t="n"/>
-      <c r="C29" s="13" t="inlineStr">
-        <is>
-          <t>Tractor Farmtrac 6075N 4WD</t>
-        </is>
-      </c>
-      <c r="D29" s="14" t="n">
-        <v>19500</v>
-      </c>
-      <c r="E29" s="18" t="n">
-        <v>16999</v>
-      </c>
-      <c r="F29" s="15">
-        <f>IF(ISNUMBER(E29),ROUND(E29*Curs,0),IF(ISNUMBER(D29),ROUND(D29*Curs,0),"La cerere"))</f>
-        <v/>
-      </c>
-      <c r="G29" s="16" t="n"/>
-      <c r="H29" s="17" t="inlineStr">
-        <is>
-          <t>Vezi pe site</t>
-        </is>
-      </c>
-      <c r="I29" s="17" t="inlineStr">
-        <is>
-          <t>Deschide oferta</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="46" customHeight="1">
-      <c r="A30" s="11" t="n">
-        <v>22</v>
-      </c>
-      <c r="B30" s="12" t="n"/>
-      <c r="C30" s="13" t="inlineStr">
-        <is>
-          <t>Tractor Farmtrac 6075N 4WD Cabină</t>
-        </is>
-      </c>
-      <c r="D30" s="14" t="n">
-        <v>24500</v>
-      </c>
-      <c r="E30" s="18" t="n">
-        <v>23000</v>
-      </c>
-      <c r="F30" s="15">
-        <f>IF(ISNUMBER(E30),ROUND(E30*Curs,0),IF(ISNUMBER(D30),ROUND(D30*Curs,0),"La cerere"))</f>
-        <v/>
-      </c>
-      <c r="G30" s="16" t="n"/>
-      <c r="H30" s="17" t="inlineStr">
-        <is>
-          <t>Vezi pe site</t>
-        </is>
-      </c>
-      <c r="I30" s="17" t="inlineStr">
-        <is>
-          <t>Deschide oferta</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  TRACTOARE ANTONIO CARRARO  ·  3 modele</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="46" customHeight="1">
-      <c r="A32" s="11" t="n">
-        <v>23</v>
-      </c>
-      <c r="B32" s="12" t="n"/>
-      <c r="C32" s="13" t="inlineStr">
-        <is>
-          <t>Tractor Antonio Carraro AV2100L</t>
-        </is>
-      </c>
-      <c r="D32" s="14" t="n">
-        <v>48000</v>
-      </c>
-      <c r="E32" s="12" t="n"/>
-      <c r="F32" s="15">
-        <f>IF(ISNUMBER(E32),ROUND(E32*Curs,0),IF(ISNUMBER(D32),ROUND(D32*Curs,0),"La cerere"))</f>
-        <v/>
-      </c>
-      <c r="G32" s="16" t="n"/>
-      <c r="H32" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I32" s="17" t="inlineStr">
-        <is>
-          <t>Deschide oferta</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="46" customHeight="1">
-      <c r="A33" s="11" t="n">
-        <v>24</v>
-      </c>
-      <c r="B33" s="12" t="n"/>
-      <c r="C33" s="13" t="inlineStr">
-        <is>
-          <t>Tractor Antonio Carraro TGF 9900</t>
-        </is>
-      </c>
-      <c r="D33" s="14" t="n">
-        <v>45000</v>
-      </c>
-      <c r="E33" s="12" t="n"/>
-      <c r="F33" s="15">
-        <f>IF(ISNUMBER(E33),ROUND(E33*Curs,0),IF(ISNUMBER(D33),ROUND(D33*Curs,0),"La cerere"))</f>
-        <v/>
-      </c>
-      <c r="G33" s="16" t="n"/>
-      <c r="H33" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I33" s="17" t="inlineStr">
-        <is>
-          <t>Deschide oferta</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="46" customHeight="1">
-      <c r="A34" s="11" t="n">
-        <v>25</v>
-      </c>
-      <c r="B34" s="12" t="n"/>
-      <c r="C34" s="13" t="inlineStr">
-        <is>
-          <t>Tractor Antonio Carraro TRG 9900</t>
-        </is>
-      </c>
-      <c r="D34" s="14" t="n">
-        <v>48000</v>
-      </c>
-      <c r="E34" s="12" t="n"/>
-      <c r="F34" s="15">
-        <f>IF(ISNUMBER(E34),ROUND(E34*Curs,0),IF(ISNUMBER(D34),ROUND(D34*Curs,0),"La cerere"))</f>
-        <v/>
-      </c>
-      <c r="G34" s="16" t="inlineStr">
-        <is>
-          <t>Reversibil</t>
-        </is>
-      </c>
-      <c r="H34" s="17" t="inlineStr">
-        <is>
-          <t>Vezi pe site</t>
-        </is>
-      </c>
-      <c r="I34" s="17" t="inlineStr">
-        <is>
-          <t>Deschide oferta</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="30" customHeight="1">
-      <c r="A35" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  TRACTOARE SOLIS  ·  8 modele</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="46" customHeight="1">
-      <c r="A36" s="11" t="n">
-        <v>26</v>
-      </c>
-      <c r="B36" s="12" t="n"/>
-      <c r="C36" s="13" t="inlineStr">
-        <is>
-          <t>Tractor Solis S16</t>
-        </is>
-      </c>
-      <c r="D36" s="14" t="n">
-        <v>6000</v>
-      </c>
-      <c r="E36" s="12" t="n"/>
-      <c r="F36" s="15">
-        <f>IF(ISNUMBER(E36),ROUND(E36*Curs,0),IF(ISNUMBER(D36),ROUND(D36*Curs,0),"La cerere"))</f>
-        <v/>
-      </c>
-      <c r="G36" s="16" t="n"/>
-      <c r="H36" s="17" t="inlineStr">
-        <is>
-          <t>Vezi pe site</t>
-        </is>
-      </c>
-      <c r="I36" s="17" t="inlineStr">
-        <is>
-          <t>Deschide oferta</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="46" customHeight="1">
-      <c r="A37" s="11" t="n">
-        <v>27</v>
-      </c>
-      <c r="B37" s="12" t="n"/>
-      <c r="C37" s="13" t="inlineStr">
-        <is>
-          <t>Tractor Solis S26</t>
-        </is>
-      </c>
-      <c r="D37" s="14" t="n">
-        <v>8000</v>
-      </c>
-      <c r="E37" s="12" t="n"/>
-      <c r="F37" s="15">
-        <f>IF(ISNUMBER(E37),ROUND(E37*Curs,0),IF(ISNUMBER(D37),ROUND(D37*Curs,0),"La cerere"))</f>
-        <v/>
-      </c>
-      <c r="G37" s="16" t="n"/>
-      <c r="H37" s="17" t="inlineStr">
-        <is>
-          <t>Vezi pe site</t>
-        </is>
-      </c>
-      <c r="I37" s="17" t="inlineStr">
-        <is>
-          <t>Deschide oferta</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="46" customHeight="1">
-      <c r="A38" s="11" t="n">
-        <v>28</v>
-      </c>
-      <c r="B38" s="12" t="n"/>
-      <c r="C38" s="13" t="inlineStr">
-        <is>
-          <t>Tractor Solis S26 Xtra</t>
-        </is>
-      </c>
-      <c r="D38" s="14" t="n">
-        <v>8300</v>
-      </c>
-      <c r="E38" s="12" t="n"/>
-      <c r="F38" s="15">
-        <f>IF(ISNUMBER(E38),ROUND(E38*Curs,0),IF(ISNUMBER(D38),ROUND(D38*Curs,0),"La cerere"))</f>
-        <v/>
-      </c>
-      <c r="G38" s="16" t="n"/>
-      <c r="H38" s="17" t="inlineStr">
-        <is>
-          <t>Vezi pe site</t>
-        </is>
-      </c>
-      <c r="I38" s="17" t="inlineStr">
-        <is>
-          <t>Deschide oferta</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="46" customHeight="1">
-      <c r="A39" s="11" t="n">
-        <v>29</v>
-      </c>
-      <c r="B39" s="12" t="n"/>
-      <c r="C39" s="13" t="inlineStr">
-        <is>
-          <t>Tractor Solis S26 Shuttle XL</t>
-        </is>
-      </c>
-      <c r="D39" s="14" t="n">
-        <v>8500</v>
-      </c>
-      <c r="E39" s="12" t="n"/>
-      <c r="F39" s="15">
-        <f>IF(ISNUMBER(E39),ROUND(E39*Curs,0),IF(ISNUMBER(D39),ROUND(D39*Curs,0),"La cerere"))</f>
-        <v/>
-      </c>
-      <c r="G39" s="16" t="n"/>
-      <c r="H39" s="17" t="inlineStr">
-        <is>
-          <t>Vezi pe site</t>
-        </is>
-      </c>
-      <c r="I39" s="17" t="inlineStr">
-        <is>
-          <t>Deschide oferta</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="46" customHeight="1">
-      <c r="A40" s="11" t="n">
-        <v>30</v>
-      </c>
-      <c r="B40" s="12" t="n"/>
-      <c r="C40" s="13" t="inlineStr">
-        <is>
-          <t>Tractor Solis S30</t>
-        </is>
-      </c>
-      <c r="D40" s="14" t="n">
-        <v>8700</v>
-      </c>
-      <c r="E40" s="12" t="n"/>
-      <c r="F40" s="15">
-        <f>IF(ISNUMBER(E40),ROUND(E40*Curs,0),IF(ISNUMBER(D40),ROUND(D40*Curs,0),"La cerere"))</f>
-        <v/>
-      </c>
-      <c r="G40" s="16" t="n"/>
-      <c r="H40" s="17" t="inlineStr">
-        <is>
-          <t>Vezi pe site</t>
-        </is>
-      </c>
-      <c r="I40" s="17" t="inlineStr">
-        <is>
-          <t>Deschide oferta</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="46" customHeight="1">
-      <c r="A41" s="11" t="n">
-        <v>31</v>
-      </c>
-      <c r="B41" s="12" t="n"/>
-      <c r="C41" s="13" t="inlineStr">
-        <is>
-          <t>Tractor Solis S32</t>
-        </is>
-      </c>
-      <c r="D41" s="14" t="n">
-        <v>9100</v>
-      </c>
-      <c r="E41" s="12" t="n"/>
-      <c r="F41" s="15">
-        <f>IF(ISNUMBER(E41),ROUND(E41*Curs,0),IF(ISNUMBER(D41),ROUND(D41*Curs,0),"La cerere"))</f>
-        <v/>
-      </c>
-      <c r="G41" s="16" t="n"/>
-      <c r="H41" s="17" t="inlineStr">
-        <is>
-          <t>Vezi pe site</t>
-        </is>
-      </c>
-      <c r="I41" s="17" t="inlineStr">
-        <is>
-          <t>Deschide oferta</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="46" customHeight="1">
-      <c r="A42" s="11" t="n">
-        <v>32</v>
-      </c>
-      <c r="B42" s="12" t="n"/>
-      <c r="C42" s="13" t="inlineStr">
-        <is>
-          <t>Tractor Solis 90N</t>
-        </is>
-      </c>
-      <c r="D42" s="14" t="n">
-        <v>29500</v>
-      </c>
-      <c r="E42" s="12" t="n"/>
-      <c r="F42" s="15">
-        <f>IF(ISNUMBER(E42),ROUND(E42*Curs,0),IF(ISNUMBER(D42),ROUND(D42*Curs,0),"La cerere"))</f>
-        <v/>
-      </c>
-      <c r="G42" s="16" t="n"/>
-      <c r="H42" s="17" t="inlineStr">
-        <is>
-          <t>Vezi pe site</t>
-        </is>
-      </c>
-      <c r="I42" s="17" t="inlineStr">
-        <is>
-          <t>Deschide oferta</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="46" customHeight="1">
-      <c r="A43" s="11" t="n">
-        <v>33</v>
-      </c>
-      <c r="B43" s="12" t="n"/>
-      <c r="C43" s="13" t="inlineStr">
-        <is>
-          <t>Tractor Solis 90RX</t>
-        </is>
-      </c>
-      <c r="D43" s="14" t="n">
-        <v>27500</v>
-      </c>
-      <c r="E43" s="12" t="n"/>
-      <c r="F43" s="15">
-        <f>IF(ISNUMBER(E43),ROUND(E43*Curs,0),IF(ISNUMBER(D43),ROUND(D43*Curs,0),"La cerere"))</f>
-        <v/>
-      </c>
-      <c r="G43" s="16" t="n"/>
-      <c r="H43" s="17" t="inlineStr">
-        <is>
-          <t>Vezi pe site</t>
-        </is>
-      </c>
-      <c r="I43" s="17" t="inlineStr">
-        <is>
-          <t>Deschide oferta</t>
+    <row r="43">
+      <c r="C43" s="19" t="inlineStr">
+        <is>
+          <t>* Preț MDL = prețul final (promo, dacă există) × cursul EUR/MDL din celula F3. Este orientativ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="C44" s="19" t="inlineStr">
+        <is>
+          <t>Cursul se poate schimba direct în F3. În Google Sheets se poate lega automat: =GOOGLEFINANCE("CURRENCY:EURMDL")</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="C45" s="20" t="inlineStr">
-        <is>
-          <t>* Preț MDL = prețul final (promo, dacă există) × cursul EUR/MDL din celula F3. Este orientativ.</t>
+      <c r="C45" s="19" t="inlineStr">
+        <is>
+          <t>Pentru o ofertă cu unul sau mai multe produse folosiți foaia „Ofertă comercială”.</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="C46" s="20" t="inlineStr">
-        <is>
-          <t>Cursul se poate schimba direct în F3. În Google Sheets se poate lega automat: =GOOGLEFINANCE("CURRENCY:EURMDL")</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="C47" s="20" t="inlineStr">
-        <is>
-          <t>Pentru o ofertă cu unul sau mai multe produse folosiți foaia „Ofertă comercială”.</t>
+      <c r="C46" s="19" t="inlineStr">
+        <is>
+          <t>„Ozonteh Impex” SRL · MD-3701, mun. Strășeni, șos. Chișinău 69, Republica Moldova · office@ozonteh.md · ozonteh.net</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A7:I7"/>
-    <mergeCell ref="A35:I35"/>
-    <mergeCell ref="A31:I31"/>
-    <mergeCell ref="A22:I22"/>
+    <mergeCell ref="A29:I29"/>
+    <mergeCell ref="A5:I5"/>
+    <mergeCell ref="A20:I20"/>
+    <mergeCell ref="A33:I33"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I41" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I42" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I43" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I41" r:id="rId64"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
@@ -3032,45 +3033,45 @@
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="D1" s="21" t="inlineStr">
+      <c r="D1" s="20" t="inlineStr">
         <is>
           <t>„Ozonteh Impex” SRL</t>
         </is>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
-      <c r="D2" s="22" t="inlineStr">
+      <c r="D2" s="21" t="inlineStr">
         <is>
           <t>MD-3701, mun. Strășeni, șos. Chișinău 69, Republica Moldova</t>
         </is>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1">
-      <c r="D3" s="22" t="inlineStr">
+      <c r="D3" s="21" t="inlineStr">
         <is>
           <t>C.F. 1013600012644 · Cod TVA 8600854</t>
         </is>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1">
-      <c r="D4" s="22" t="inlineStr">
+      <c r="D4" s="21" t="inlineStr">
         <is>
           <t>office@ozonteh.md · ozonteh.net</t>
         </is>
       </c>
     </row>
     <row r="5" ht="8" customHeight="1">
-      <c r="A5" s="23" t="n"/>
-      <c r="B5" s="23" t="n"/>
-      <c r="C5" s="23" t="n"/>
-      <c r="D5" s="23" t="n"/>
-      <c r="E5" s="23" t="n"/>
-      <c r="F5" s="23" t="n"/>
-      <c r="G5" s="23" t="n"/>
-      <c r="H5" s="23" t="n"/>
+      <c r="A5" s="22" t="n"/>
+      <c r="B5" s="22" t="n"/>
+      <c r="C5" s="22" t="n"/>
+      <c r="D5" s="22" t="n"/>
+      <c r="E5" s="22" t="n"/>
+      <c r="F5" s="22" t="n"/>
+      <c r="G5" s="22" t="n"/>
+      <c r="H5" s="22" t="n"/>
     </row>
     <row r="7" ht="32" customHeight="1">
-      <c r="A7" s="24" t="inlineStr">
+      <c r="A7" s="23" t="inlineStr">
         <is>
           <t>OFERTĂ COMERCIALĂ</t>
         </is>
@@ -3082,20 +3083,20 @@
           <t>Nr. ofertei:</t>
         </is>
       </c>
-      <c r="C8" s="25" t="n"/>
-      <c r="D8" s="26" t="n"/>
+      <c r="C8" s="24" t="n"/>
+      <c r="D8" s="25" t="n"/>
       <c r="E8" s="4" t="inlineStr">
         <is>
           <t>Data:</t>
         </is>
       </c>
-      <c r="F8" s="27" t="n"/>
+      <c r="F8" s="26" t="n"/>
       <c r="G8" s="4" t="inlineStr">
         <is>
           <t>Valabilă (zile):</t>
         </is>
       </c>
-      <c r="H8" s="28" t="n">
+      <c r="H8" s="27" t="n">
         <v>14</v>
       </c>
     </row>
@@ -3105,17 +3106,17 @@
           <t>Curs EUR/MDL:</t>
         </is>
       </c>
-      <c r="C9" s="29">
+      <c r="C9" s="28">
         <f>Curs</f>
         <v/>
       </c>
-      <c r="D9" s="26" t="n"/>
+      <c r="D9" s="25" t="n"/>
       <c r="E9" s="4" t="inlineStr">
         <is>
           <t>Cota TVA:</t>
         </is>
       </c>
-      <c r="F9" s="30" t="n">
+      <c r="F9" s="29" t="n">
         <v>0.2</v>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -3123,128 +3124,128 @@
           <t>Expiră la:</t>
         </is>
       </c>
-      <c r="H9" s="31">
+      <c r="H9" s="30">
         <f>IF(ISNUMBER(F8),F8+H8,"")</f>
         <v/>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="32" t="inlineStr">
+      <c r="A11" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">  DATE CLIENT</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="B12" s="33" t="inlineStr">
+      <c r="B12" s="32" t="inlineStr">
         <is>
           <t>Client / companie:</t>
         </is>
       </c>
-      <c r="C12" s="34" t="n"/>
-      <c r="D12" s="26" t="n"/>
-      <c r="E12" s="26" t="n"/>
-      <c r="F12" s="26" t="n"/>
-      <c r="G12" s="26" t="n"/>
-      <c r="H12" s="26" t="n"/>
+      <c r="C12" s="33" t="n"/>
+      <c r="D12" s="25" t="n"/>
+      <c r="E12" s="25" t="n"/>
+      <c r="F12" s="25" t="n"/>
+      <c r="G12" s="25" t="n"/>
+      <c r="H12" s="25" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="B13" s="33" t="inlineStr">
+      <c r="B13" s="32" t="inlineStr">
         <is>
           <t>Persoană de contact:</t>
         </is>
       </c>
-      <c r="C13" s="34" t="n"/>
-      <c r="D13" s="26" t="n"/>
-      <c r="E13" s="26" t="n"/>
-      <c r="F13" s="26" t="n"/>
-      <c r="G13" s="26" t="n"/>
-      <c r="H13" s="26" t="n"/>
+      <c r="C13" s="33" t="n"/>
+      <c r="D13" s="25" t="n"/>
+      <c r="E13" s="25" t="n"/>
+      <c r="F13" s="25" t="n"/>
+      <c r="G13" s="25" t="n"/>
+      <c r="H13" s="25" t="n"/>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="B14" s="33" t="inlineStr">
+      <c r="B14" s="32" t="inlineStr">
         <is>
           <t>Telefon:</t>
         </is>
       </c>
-      <c r="C14" s="34" t="n"/>
-      <c r="D14" s="26" t="n"/>
+      <c r="C14" s="33" t="n"/>
+      <c r="D14" s="25" t="n"/>
       <c r="E14" s="4" t="inlineStr">
         <is>
           <t>E-mail:</t>
         </is>
       </c>
-      <c r="F14" s="34" t="n"/>
-      <c r="G14" s="26" t="n"/>
-      <c r="H14" s="26" t="n"/>
+      <c r="F14" s="33" t="n"/>
+      <c r="G14" s="25" t="n"/>
+      <c r="H14" s="25" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="B15" s="33" t="inlineStr">
+      <c r="B15" s="32" t="inlineStr">
         <is>
           <t>Localitate / adresă:</t>
         </is>
       </c>
-      <c r="C15" s="34" t="n"/>
-      <c r="D15" s="26" t="n"/>
-      <c r="E15" s="26" t="n"/>
-      <c r="F15" s="26" t="n"/>
-      <c r="G15" s="26" t="n"/>
-      <c r="H15" s="26" t="n"/>
+      <c r="C15" s="33" t="n"/>
+      <c r="D15" s="25" t="n"/>
+      <c r="E15" s="25" t="n"/>
+      <c r="F15" s="25" t="n"/>
+      <c r="G15" s="25" t="n"/>
+      <c r="H15" s="25" t="n"/>
     </row>
     <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="32" t="inlineStr">
+      <c r="A17" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">  PRODUSE OFERITE</t>
         </is>
       </c>
     </row>
     <row r="18" ht="32" customHeight="1">
-      <c r="A18" s="35" t="inlineStr">
+      <c r="A18" s="34" t="inlineStr">
         <is>
           <t>Nr.</t>
         </is>
       </c>
-      <c r="B18" s="35" t="inlineStr">
+      <c r="B18" s="34" t="inlineStr">
         <is>
           <t>Produs (alegeți din listă)</t>
         </is>
       </c>
-      <c r="C18" s="35" t="inlineStr">
+      <c r="C18" s="34" t="inlineStr">
         <is>
           <t>Pagina
 produsului</t>
         </is>
       </c>
-      <c r="D18" s="35" t="inlineStr">
+      <c r="D18" s="34" t="inlineStr">
         <is>
           <t>Cant.</t>
         </is>
       </c>
-      <c r="E18" s="35" t="inlineStr">
+      <c r="E18" s="34" t="inlineStr">
         <is>
           <t>Preț unitar
 EUR fără TVA</t>
         </is>
       </c>
-      <c r="F18" s="35" t="inlineStr">
+      <c r="F18" s="34" t="inlineStr">
         <is>
           <t>Reducere
 %</t>
         </is>
       </c>
-      <c r="G18" s="35" t="inlineStr">
+      <c r="G18" s="34" t="inlineStr">
         <is>
           <t>Total EUR
 fără TVA</t>
         </is>
       </c>
-      <c r="H18" s="35" t="inlineStr">
+      <c r="H18" s="34" t="inlineStr">
         <is>
           <t>Total MDL
 fără TVA</t>
         </is>
       </c>
-      <c r="I18" s="7" t="inlineStr">
+      <c r="I18" s="35" t="inlineStr">
         <is>
           <t>Link ofertă produs (pentru meniul Ozonteh)</t>
         </is>
@@ -3264,14 +3265,14 @@
         <f>IF(B19="","",IFERROR(HYPERLINK(INDEX(Catalog!$B$2:$B$34,MATCH(B19,Catalog!$A$2:$A$34,0)),"Vezi produs"),""))</f>
         <v/>
       </c>
-      <c r="D19" s="25" t="n">
+      <c r="D19" s="24" t="n">
         <v>1</v>
       </c>
       <c r="E19" s="39">
         <f>IF(B19="","",IFERROR(INDEX(Catalog!$C$2:$C$34,MATCH(B19,Catalog!$A$2:$A$34,0)),"nu e în listă"))</f>
         <v/>
       </c>
-      <c r="F19" s="30" t="n"/>
+      <c r="F19" s="29" t="n"/>
       <c r="G19" s="40">
         <f>IF(AND(ISNUMBER(D19),ISNUMBER(E19)),ROUND(D19*E19*(1-N(F19)),2),"")</f>
         <v/>
@@ -3280,7 +3281,7 @@
         <f>IF(ISNUMBER(G19),ROUND(G19*$C$9,0),"")</f>
         <v/>
       </c>
-      <c r="I19" s="7">
+      <c r="I19" s="35">
         <f>IF(B19="","",IFERROR(INDEX(Catalog!$F$2:$F$34,MATCH(B19,Catalog!$A$2:$A$34,0))&amp;"",""))</f>
         <v/>
       </c>
@@ -3295,12 +3296,12 @@
         <f>IF(B20="","",IFERROR(HYPERLINK(INDEX(Catalog!$B$2:$B$34,MATCH(B20,Catalog!$A$2:$A$34,0)),"Vezi produs"),""))</f>
         <v/>
       </c>
-      <c r="D20" s="25" t="n"/>
+      <c r="D20" s="24" t="n"/>
       <c r="E20" s="39">
         <f>IF(B20="","",IFERROR(INDEX(Catalog!$C$2:$C$34,MATCH(B20,Catalog!$A$2:$A$34,0)),"nu e în listă"))</f>
         <v/>
       </c>
-      <c r="F20" s="30" t="n"/>
+      <c r="F20" s="29" t="n"/>
       <c r="G20" s="40">
         <f>IF(AND(ISNUMBER(D20),ISNUMBER(E20)),ROUND(D20*E20*(1-N(F20)),2),"")</f>
         <v/>
@@ -3309,7 +3310,7 @@
         <f>IF(ISNUMBER(G20),ROUND(G20*$C$9,0),"")</f>
         <v/>
       </c>
-      <c r="I20" s="7">
+      <c r="I20" s="35">
         <f>IF(B20="","",IFERROR(INDEX(Catalog!$F$2:$F$34,MATCH(B20,Catalog!$A$2:$A$34,0))&amp;"",""))</f>
         <v/>
       </c>
@@ -3324,12 +3325,12 @@
         <f>IF(B21="","",IFERROR(HYPERLINK(INDEX(Catalog!$B$2:$B$34,MATCH(B21,Catalog!$A$2:$A$34,0)),"Vezi produs"),""))</f>
         <v/>
       </c>
-      <c r="D21" s="25" t="n"/>
+      <c r="D21" s="24" t="n"/>
       <c r="E21" s="39">
         <f>IF(B21="","",IFERROR(INDEX(Catalog!$C$2:$C$34,MATCH(B21,Catalog!$A$2:$A$34,0)),"nu e în listă"))</f>
         <v/>
       </c>
-      <c r="F21" s="30" t="n"/>
+      <c r="F21" s="29" t="n"/>
       <c r="G21" s="40">
         <f>IF(AND(ISNUMBER(D21),ISNUMBER(E21)),ROUND(D21*E21*(1-N(F21)),2),"")</f>
         <v/>
@@ -3338,7 +3339,7 @@
         <f>IF(ISNUMBER(G21),ROUND(G21*$C$9,0),"")</f>
         <v/>
       </c>
-      <c r="I21" s="7">
+      <c r="I21" s="35">
         <f>IF(B21="","",IFERROR(INDEX(Catalog!$F$2:$F$34,MATCH(B21,Catalog!$A$2:$A$34,0))&amp;"",""))</f>
         <v/>
       </c>
@@ -3353,12 +3354,12 @@
         <f>IF(B22="","",IFERROR(HYPERLINK(INDEX(Catalog!$B$2:$B$34,MATCH(B22,Catalog!$A$2:$A$34,0)),"Vezi produs"),""))</f>
         <v/>
       </c>
-      <c r="D22" s="25" t="n"/>
+      <c r="D22" s="24" t="n"/>
       <c r="E22" s="39">
         <f>IF(B22="","",IFERROR(INDEX(Catalog!$C$2:$C$34,MATCH(B22,Catalog!$A$2:$A$34,0)),"nu e în listă"))</f>
         <v/>
       </c>
-      <c r="F22" s="30" t="n"/>
+      <c r="F22" s="29" t="n"/>
       <c r="G22" s="40">
         <f>IF(AND(ISNUMBER(D22),ISNUMBER(E22)),ROUND(D22*E22*(1-N(F22)),2),"")</f>
         <v/>
@@ -3367,7 +3368,7 @@
         <f>IF(ISNUMBER(G22),ROUND(G22*$C$9,0),"")</f>
         <v/>
       </c>
-      <c r="I22" s="7">
+      <c r="I22" s="35">
         <f>IF(B22="","",IFERROR(INDEX(Catalog!$F$2:$F$34,MATCH(B22,Catalog!$A$2:$A$34,0))&amp;"",""))</f>
         <v/>
       </c>
@@ -3382,12 +3383,12 @@
         <f>IF(B23="","",IFERROR(HYPERLINK(INDEX(Catalog!$B$2:$B$34,MATCH(B23,Catalog!$A$2:$A$34,0)),"Vezi produs"),""))</f>
         <v/>
       </c>
-      <c r="D23" s="25" t="n"/>
+      <c r="D23" s="24" t="n"/>
       <c r="E23" s="39">
         <f>IF(B23="","",IFERROR(INDEX(Catalog!$C$2:$C$34,MATCH(B23,Catalog!$A$2:$A$34,0)),"nu e în listă"))</f>
         <v/>
       </c>
-      <c r="F23" s="30" t="n"/>
+      <c r="F23" s="29" t="n"/>
       <c r="G23" s="40">
         <f>IF(AND(ISNUMBER(D23),ISNUMBER(E23)),ROUND(D23*E23*(1-N(F23)),2),"")</f>
         <v/>
@@ -3396,7 +3397,7 @@
         <f>IF(ISNUMBER(G23),ROUND(G23*$C$9,0),"")</f>
         <v/>
       </c>
-      <c r="I23" s="7">
+      <c r="I23" s="35">
         <f>IF(B23="","",IFERROR(INDEX(Catalog!$F$2:$F$34,MATCH(B23,Catalog!$A$2:$A$34,0))&amp;"",""))</f>
         <v/>
       </c>
@@ -3411,12 +3412,12 @@
         <f>IF(B24="","",IFERROR(HYPERLINK(INDEX(Catalog!$B$2:$B$34,MATCH(B24,Catalog!$A$2:$A$34,0)),"Vezi produs"),""))</f>
         <v/>
       </c>
-      <c r="D24" s="25" t="n"/>
+      <c r="D24" s="24" t="n"/>
       <c r="E24" s="39">
         <f>IF(B24="","",IFERROR(INDEX(Catalog!$C$2:$C$34,MATCH(B24,Catalog!$A$2:$A$34,0)),"nu e în listă"))</f>
         <v/>
       </c>
-      <c r="F24" s="30" t="n"/>
+      <c r="F24" s="29" t="n"/>
       <c r="G24" s="40">
         <f>IF(AND(ISNUMBER(D24),ISNUMBER(E24)),ROUND(D24*E24*(1-N(F24)),2),"")</f>
         <v/>
@@ -3425,7 +3426,7 @@
         <f>IF(ISNUMBER(G24),ROUND(G24*$C$9,0),"")</f>
         <v/>
       </c>
-      <c r="I24" s="7">
+      <c r="I24" s="35">
         <f>IF(B24="","",IFERROR(INDEX(Catalog!$F$2:$F$34,MATCH(B24,Catalog!$A$2:$A$34,0))&amp;"",""))</f>
         <v/>
       </c>
@@ -3440,12 +3441,12 @@
         <f>IF(B25="","",IFERROR(HYPERLINK(INDEX(Catalog!$B$2:$B$34,MATCH(B25,Catalog!$A$2:$A$34,0)),"Vezi produs"),""))</f>
         <v/>
       </c>
-      <c r="D25" s="25" t="n"/>
+      <c r="D25" s="24" t="n"/>
       <c r="E25" s="39">
         <f>IF(B25="","",IFERROR(INDEX(Catalog!$C$2:$C$34,MATCH(B25,Catalog!$A$2:$A$34,0)),"nu e în listă"))</f>
         <v/>
       </c>
-      <c r="F25" s="30" t="n"/>
+      <c r="F25" s="29" t="n"/>
       <c r="G25" s="40">
         <f>IF(AND(ISNUMBER(D25),ISNUMBER(E25)),ROUND(D25*E25*(1-N(F25)),2),"")</f>
         <v/>
@@ -3454,7 +3455,7 @@
         <f>IF(ISNUMBER(G25),ROUND(G25*$C$9,0),"")</f>
         <v/>
       </c>
-      <c r="I25" s="7">
+      <c r="I25" s="35">
         <f>IF(B25="","",IFERROR(INDEX(Catalog!$F$2:$F$34,MATCH(B25,Catalog!$A$2:$A$34,0))&amp;"",""))</f>
         <v/>
       </c>
@@ -3469,12 +3470,12 @@
         <f>IF(B26="","",IFERROR(HYPERLINK(INDEX(Catalog!$B$2:$B$34,MATCH(B26,Catalog!$A$2:$A$34,0)),"Vezi produs"),""))</f>
         <v/>
       </c>
-      <c r="D26" s="25" t="n"/>
+      <c r="D26" s="24" t="n"/>
       <c r="E26" s="39">
         <f>IF(B26="","",IFERROR(INDEX(Catalog!$C$2:$C$34,MATCH(B26,Catalog!$A$2:$A$34,0)),"nu e în listă"))</f>
         <v/>
       </c>
-      <c r="F26" s="30" t="n"/>
+      <c r="F26" s="29" t="n"/>
       <c r="G26" s="40">
         <f>IF(AND(ISNUMBER(D26),ISNUMBER(E26)),ROUND(D26*E26*(1-N(F26)),2),"")</f>
         <v/>
@@ -3483,7 +3484,7 @@
         <f>IF(ISNUMBER(G26),ROUND(G26*$C$9,0),"")</f>
         <v/>
       </c>
-      <c r="I26" s="7">
+      <c r="I26" s="35">
         <f>IF(B26="","",IFERROR(INDEX(Catalog!$F$2:$F$34,MATCH(B26,Catalog!$A$2:$A$34,0))&amp;"",""))</f>
         <v/>
       </c>
@@ -3498,12 +3499,12 @@
         <f>IF(B27="","",IFERROR(HYPERLINK(INDEX(Catalog!$B$2:$B$34,MATCH(B27,Catalog!$A$2:$A$34,0)),"Vezi produs"),""))</f>
         <v/>
       </c>
-      <c r="D27" s="25" t="n"/>
+      <c r="D27" s="24" t="n"/>
       <c r="E27" s="39">
         <f>IF(B27="","",IFERROR(INDEX(Catalog!$C$2:$C$34,MATCH(B27,Catalog!$A$2:$A$34,0)),"nu e în listă"))</f>
         <v/>
       </c>
-      <c r="F27" s="30" t="n"/>
+      <c r="F27" s="29" t="n"/>
       <c r="G27" s="40">
         <f>IF(AND(ISNUMBER(D27),ISNUMBER(E27)),ROUND(D27*E27*(1-N(F27)),2),"")</f>
         <v/>
@@ -3512,7 +3513,7 @@
         <f>IF(ISNUMBER(G27),ROUND(G27*$C$9,0),"")</f>
         <v/>
       </c>
-      <c r="I27" s="7">
+      <c r="I27" s="35">
         <f>IF(B27="","",IFERROR(INDEX(Catalog!$F$2:$F$34,MATCH(B27,Catalog!$A$2:$A$34,0))&amp;"",""))</f>
         <v/>
       </c>
@@ -3527,12 +3528,12 @@
         <f>IF(B28="","",IFERROR(HYPERLINK(INDEX(Catalog!$B$2:$B$34,MATCH(B28,Catalog!$A$2:$A$34,0)),"Vezi produs"),""))</f>
         <v/>
       </c>
-      <c r="D28" s="25" t="n"/>
+      <c r="D28" s="24" t="n"/>
       <c r="E28" s="39">
         <f>IF(B28="","",IFERROR(INDEX(Catalog!$C$2:$C$34,MATCH(B28,Catalog!$A$2:$A$34,0)),"nu e în listă"))</f>
         <v/>
       </c>
-      <c r="F28" s="30" t="n"/>
+      <c r="F28" s="29" t="n"/>
       <c r="G28" s="40">
         <f>IF(AND(ISNUMBER(D28),ISNUMBER(E28)),ROUND(D28*E28*(1-N(F28)),2),"")</f>
         <v/>
@@ -3541,7 +3542,7 @@
         <f>IF(ISNUMBER(G28),ROUND(G28*$C$9,0),"")</f>
         <v/>
       </c>
-      <c r="I28" s="7">
+      <c r="I28" s="35">
         <f>IF(B28="","",IFERROR(INDEX(Catalog!$F$2:$F$34,MATCH(B28,Catalog!$A$2:$A$34,0))&amp;"",""))</f>
         <v/>
       </c>
@@ -3591,14 +3592,14 @@
       </c>
     </row>
     <row r="34" ht="22" customHeight="1">
-      <c r="A34" s="32" t="inlineStr">
+      <c r="A34" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">  CONDIȚII</t>
         </is>
       </c>
     </row>
     <row r="35" ht="20" customHeight="1">
-      <c r="B35" s="33" t="inlineStr">
+      <c r="B35" s="32" t="inlineStr">
         <is>
           <t>Garanție:</t>
         </is>
@@ -3610,7 +3611,7 @@
       </c>
     </row>
     <row r="36" ht="20" customHeight="1">
-      <c r="B36" s="33" t="inlineStr">
+      <c r="B36" s="32" t="inlineStr">
         <is>
           <t>Livrare:</t>
         </is>
@@ -3622,7 +3623,7 @@
       </c>
     </row>
     <row r="37" ht="20" customHeight="1">
-      <c r="B37" s="33" t="inlineStr">
+      <c r="B37" s="32" t="inlineStr">
         <is>
           <t>Finanțare:</t>
         </is>
@@ -3634,7 +3635,7 @@
       </c>
     </row>
     <row r="38" ht="20" customHeight="1">
-      <c r="B38" s="33" t="inlineStr">
+      <c r="B38" s="32" t="inlineStr">
         <is>
           <t>Service:</t>
         </is>
@@ -3646,7 +3647,7 @@
       </c>
     </row>
     <row r="39" ht="20" customHeight="1">
-      <c r="B39" s="33" t="inlineStr">
+      <c r="B39" s="32" t="inlineStr">
         <is>
           <t>Suport post-vânzare:</t>
         </is>
@@ -3658,7 +3659,7 @@
       </c>
     </row>
     <row r="40" ht="20" customHeight="1">
-      <c r="B40" s="33" t="inlineStr">
+      <c r="B40" s="32" t="inlineStr">
         <is>
           <t>Prețuri:</t>
         </is>
@@ -3670,37 +3671,37 @@
       </c>
     </row>
     <row r="41" ht="20" customHeight="1">
-      <c r="B41" s="33" t="inlineStr">
+      <c r="B41" s="32" t="inlineStr">
         <is>
           <t>Condiții de plată:</t>
         </is>
       </c>
-      <c r="C41" s="34" t="n"/>
-      <c r="D41" s="26" t="n"/>
-      <c r="E41" s="26" t="n"/>
-      <c r="F41" s="26" t="n"/>
-      <c r="G41" s="26" t="n"/>
-      <c r="H41" s="26" t="n"/>
+      <c r="C41" s="33" t="n"/>
+      <c r="D41" s="25" t="n"/>
+      <c r="E41" s="25" t="n"/>
+      <c r="F41" s="25" t="n"/>
+      <c r="G41" s="25" t="n"/>
+      <c r="H41" s="25" t="n"/>
     </row>
     <row r="43" ht="20" customHeight="1">
-      <c r="B43" s="33" t="inlineStr">
+      <c r="B43" s="32" t="inlineStr">
         <is>
           <t>Întocmit de:</t>
         </is>
       </c>
-      <c r="C43" s="34" t="n"/>
-      <c r="D43" s="26" t="n"/>
+      <c r="C43" s="33" t="n"/>
+      <c r="D43" s="25" t="n"/>
       <c r="E43" s="4" t="inlineStr">
         <is>
           <t>Telefon:</t>
         </is>
       </c>
-      <c r="F43" s="34" t="n"/>
-      <c r="G43" s="26" t="n"/>
-      <c r="H43" s="26" t="n"/>
+      <c r="F43" s="33" t="n"/>
+      <c r="G43" s="25" t="n"/>
+      <c r="H43" s="25" t="n"/>
     </row>
     <row r="45" ht="26" customHeight="1">
-      <c r="B45" s="33" t="inlineStr">
+      <c r="B45" s="32" t="inlineStr">
         <is>
           <t>Semnătura:</t>
         </is>
@@ -4148,7 +4149,7 @@
     </row>
     <row r="2">
       <c r="A2">
-        <f>'Lista de prețuri'!C8</f>
+        <f>'Lista de prețuri'!C6</f>
         <v/>
       </c>
       <c r="B2" t="inlineStr">
@@ -4157,15 +4158,15 @@
         </is>
       </c>
       <c r="C2">
-        <f>IF(ISNUMBER('Lista de prețuri'!E8),'Lista de prețuri'!E8,IF(ISNUMBER('Lista de prețuri'!D8),'Lista de prețuri'!D8,"La cerere"))</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E6),'Lista de prețuri'!E6,IF(ISNUMBER('Lista de prețuri'!D6),'Lista de prețuri'!D6,"La cerere"))</f>
         <v/>
       </c>
       <c r="D2">
-        <f>'Lista de prețuri'!D8</f>
+        <f>'Lista de prețuri'!D6</f>
         <v/>
       </c>
       <c r="E2">
-        <f>IF(ISNUMBER('Lista de prețuri'!E8),'Lista de prețuri'!E8,"")</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E6),'Lista de prețuri'!E6,"")</f>
         <v/>
       </c>
       <c r="F2" t="inlineStr">
@@ -4181,7 +4182,7 @@
     </row>
     <row r="3">
       <c r="A3">
-        <f>'Lista de prețuri'!C9</f>
+        <f>'Lista de prețuri'!C7</f>
         <v/>
       </c>
       <c r="B3" t="inlineStr">
@@ -4190,15 +4191,15 @@
         </is>
       </c>
       <c r="C3">
-        <f>IF(ISNUMBER('Lista de prețuri'!E9),'Lista de prețuri'!E9,IF(ISNUMBER('Lista de prețuri'!D9),'Lista de prețuri'!D9,"La cerere"))</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E7),'Lista de prețuri'!E7,IF(ISNUMBER('Lista de prețuri'!D7),'Lista de prețuri'!D7,"La cerere"))</f>
         <v/>
       </c>
       <c r="D3">
-        <f>'Lista de prețuri'!D9</f>
+        <f>'Lista de prețuri'!D7</f>
         <v/>
       </c>
       <c r="E3">
-        <f>IF(ISNUMBER('Lista de prețuri'!E9),'Lista de prețuri'!E9,"")</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E7),'Lista de prețuri'!E7,"")</f>
         <v/>
       </c>
       <c r="F3" t="inlineStr">
@@ -4214,7 +4215,7 @@
     </row>
     <row r="4">
       <c r="A4">
-        <f>'Lista de prețuri'!C10</f>
+        <f>'Lista de prețuri'!C8</f>
         <v/>
       </c>
       <c r="B4" t="inlineStr">
@@ -4223,15 +4224,15 @@
         </is>
       </c>
       <c r="C4">
-        <f>IF(ISNUMBER('Lista de prețuri'!E10),'Lista de prețuri'!E10,IF(ISNUMBER('Lista de prețuri'!D10),'Lista de prețuri'!D10,"La cerere"))</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E8),'Lista de prețuri'!E8,IF(ISNUMBER('Lista de prețuri'!D8),'Lista de prețuri'!D8,"La cerere"))</f>
         <v/>
       </c>
       <c r="D4">
-        <f>'Lista de prețuri'!D10</f>
+        <f>'Lista de prețuri'!D8</f>
         <v/>
       </c>
       <c r="E4">
-        <f>IF(ISNUMBER('Lista de prețuri'!E10),'Lista de prețuri'!E10,"")</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E8),'Lista de prețuri'!E8,"")</f>
         <v/>
       </c>
       <c r="F4" t="inlineStr">
@@ -4247,7 +4248,7 @@
     </row>
     <row r="5">
       <c r="A5">
-        <f>'Lista de prețuri'!C11</f>
+        <f>'Lista de prețuri'!C9</f>
         <v/>
       </c>
       <c r="B5" t="inlineStr">
@@ -4256,15 +4257,15 @@
         </is>
       </c>
       <c r="C5">
-        <f>IF(ISNUMBER('Lista de prețuri'!E11),'Lista de prețuri'!E11,IF(ISNUMBER('Lista de prețuri'!D11),'Lista de prețuri'!D11,"La cerere"))</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E9),'Lista de prețuri'!E9,IF(ISNUMBER('Lista de prețuri'!D9),'Lista de prețuri'!D9,"La cerere"))</f>
         <v/>
       </c>
       <c r="D5">
-        <f>'Lista de prețuri'!D11</f>
+        <f>'Lista de prețuri'!D9</f>
         <v/>
       </c>
       <c r="E5">
-        <f>IF(ISNUMBER('Lista de prețuri'!E11),'Lista de prețuri'!E11,"")</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E9),'Lista de prețuri'!E9,"")</f>
         <v/>
       </c>
       <c r="F5" t="inlineStr">
@@ -4280,7 +4281,7 @@
     </row>
     <row r="6">
       <c r="A6">
-        <f>'Lista de prețuri'!C12</f>
+        <f>'Lista de prețuri'!C10</f>
         <v/>
       </c>
       <c r="B6" t="inlineStr">
@@ -4289,15 +4290,15 @@
         </is>
       </c>
       <c r="C6">
-        <f>IF(ISNUMBER('Lista de prețuri'!E12),'Lista de prețuri'!E12,IF(ISNUMBER('Lista de prețuri'!D12),'Lista de prețuri'!D12,"La cerere"))</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E10),'Lista de prețuri'!E10,IF(ISNUMBER('Lista de prețuri'!D10),'Lista de prețuri'!D10,"La cerere"))</f>
         <v/>
       </c>
       <c r="D6">
-        <f>'Lista de prețuri'!D12</f>
+        <f>'Lista de prețuri'!D10</f>
         <v/>
       </c>
       <c r="E6">
-        <f>IF(ISNUMBER('Lista de prețuri'!E12),'Lista de prețuri'!E12,"")</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E10),'Lista de prețuri'!E10,"")</f>
         <v/>
       </c>
       <c r="F6" t="inlineStr">
@@ -4313,7 +4314,7 @@
     </row>
     <row r="7">
       <c r="A7">
-        <f>'Lista de prețuri'!C13</f>
+        <f>'Lista de prețuri'!C11</f>
         <v/>
       </c>
       <c r="B7" t="inlineStr">
@@ -4322,15 +4323,15 @@
         </is>
       </c>
       <c r="C7">
-        <f>IF(ISNUMBER('Lista de prețuri'!E13),'Lista de prețuri'!E13,IF(ISNUMBER('Lista de prețuri'!D13),'Lista de prețuri'!D13,"La cerere"))</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E11),'Lista de prețuri'!E11,IF(ISNUMBER('Lista de prețuri'!D11),'Lista de prețuri'!D11,"La cerere"))</f>
         <v/>
       </c>
       <c r="D7">
-        <f>'Lista de prețuri'!D13</f>
+        <f>'Lista de prețuri'!D11</f>
         <v/>
       </c>
       <c r="E7">
-        <f>IF(ISNUMBER('Lista de prețuri'!E13),'Lista de prețuri'!E13,"")</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E11),'Lista de prețuri'!E11,"")</f>
         <v/>
       </c>
       <c r="F7" t="inlineStr">
@@ -4346,7 +4347,7 @@
     </row>
     <row r="8">
       <c r="A8">
-        <f>'Lista de prețuri'!C14</f>
+        <f>'Lista de prețuri'!C12</f>
         <v/>
       </c>
       <c r="B8" t="inlineStr">
@@ -4355,15 +4356,15 @@
         </is>
       </c>
       <c r="C8">
-        <f>IF(ISNUMBER('Lista de prețuri'!E14),'Lista de prețuri'!E14,IF(ISNUMBER('Lista de prețuri'!D14),'Lista de prețuri'!D14,"La cerere"))</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E12),'Lista de prețuri'!E12,IF(ISNUMBER('Lista de prețuri'!D12),'Lista de prețuri'!D12,"La cerere"))</f>
         <v/>
       </c>
       <c r="D8">
-        <f>'Lista de prețuri'!D14</f>
+        <f>'Lista de prețuri'!D12</f>
         <v/>
       </c>
       <c r="E8">
-        <f>IF(ISNUMBER('Lista de prețuri'!E14),'Lista de prețuri'!E14,"")</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E12),'Lista de prețuri'!E12,"")</f>
         <v/>
       </c>
       <c r="F8" t="inlineStr">
@@ -4379,7 +4380,7 @@
     </row>
     <row r="9">
       <c r="A9">
-        <f>'Lista de prețuri'!C15</f>
+        <f>'Lista de prețuri'!C13</f>
         <v/>
       </c>
       <c r="B9" t="inlineStr">
@@ -4388,15 +4389,15 @@
         </is>
       </c>
       <c r="C9">
-        <f>IF(ISNUMBER('Lista de prețuri'!E15),'Lista de prețuri'!E15,IF(ISNUMBER('Lista de prețuri'!D15),'Lista de prețuri'!D15,"La cerere"))</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E13),'Lista de prețuri'!E13,IF(ISNUMBER('Lista de prețuri'!D13),'Lista de prețuri'!D13,"La cerere"))</f>
         <v/>
       </c>
       <c r="D9">
-        <f>'Lista de prețuri'!D15</f>
+        <f>'Lista de prețuri'!D13</f>
         <v/>
       </c>
       <c r="E9">
-        <f>IF(ISNUMBER('Lista de prețuri'!E15),'Lista de prețuri'!E15,"")</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E13),'Lista de prețuri'!E13,"")</f>
         <v/>
       </c>
       <c r="F9" t="inlineStr">
@@ -4412,7 +4413,7 @@
     </row>
     <row r="10">
       <c r="A10">
-        <f>'Lista de prețuri'!C16</f>
+        <f>'Lista de prețuri'!C14</f>
         <v/>
       </c>
       <c r="B10" t="inlineStr">
@@ -4421,15 +4422,15 @@
         </is>
       </c>
       <c r="C10">
-        <f>IF(ISNUMBER('Lista de prețuri'!E16),'Lista de prețuri'!E16,IF(ISNUMBER('Lista de prețuri'!D16),'Lista de prețuri'!D16,"La cerere"))</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E14),'Lista de prețuri'!E14,IF(ISNUMBER('Lista de prețuri'!D14),'Lista de prețuri'!D14,"La cerere"))</f>
         <v/>
       </c>
       <c r="D10">
-        <f>'Lista de prețuri'!D16</f>
+        <f>'Lista de prețuri'!D14</f>
         <v/>
       </c>
       <c r="E10">
-        <f>IF(ISNUMBER('Lista de prețuri'!E16),'Lista de prețuri'!E16,"")</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E14),'Lista de prețuri'!E14,"")</f>
         <v/>
       </c>
       <c r="F10" t="inlineStr">
@@ -4445,7 +4446,7 @@
     </row>
     <row r="11">
       <c r="A11">
-        <f>'Lista de prețuri'!C17</f>
+        <f>'Lista de prețuri'!C15</f>
         <v/>
       </c>
       <c r="B11" t="inlineStr">
@@ -4454,15 +4455,15 @@
         </is>
       </c>
       <c r="C11">
-        <f>IF(ISNUMBER('Lista de prețuri'!E17),'Lista de prețuri'!E17,IF(ISNUMBER('Lista de prețuri'!D17),'Lista de prețuri'!D17,"La cerere"))</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E15),'Lista de prețuri'!E15,IF(ISNUMBER('Lista de prețuri'!D15),'Lista de prețuri'!D15,"La cerere"))</f>
         <v/>
       </c>
       <c r="D11">
-        <f>'Lista de prețuri'!D17</f>
+        <f>'Lista de prețuri'!D15</f>
         <v/>
       </c>
       <c r="E11">
-        <f>IF(ISNUMBER('Lista de prețuri'!E17),'Lista de prețuri'!E17,"")</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E15),'Lista de prețuri'!E15,"")</f>
         <v/>
       </c>
       <c r="F11" t="inlineStr">
@@ -4478,7 +4479,7 @@
     </row>
     <row r="12">
       <c r="A12">
-        <f>'Lista de prețuri'!C18</f>
+        <f>'Lista de prețuri'!C16</f>
         <v/>
       </c>
       <c r="B12" t="inlineStr">
@@ -4487,15 +4488,15 @@
         </is>
       </c>
       <c r="C12">
-        <f>IF(ISNUMBER('Lista de prețuri'!E18),'Lista de prețuri'!E18,IF(ISNUMBER('Lista de prețuri'!D18),'Lista de prețuri'!D18,"La cerere"))</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E16),'Lista de prețuri'!E16,IF(ISNUMBER('Lista de prețuri'!D16),'Lista de prețuri'!D16,"La cerere"))</f>
         <v/>
       </c>
       <c r="D12">
-        <f>'Lista de prețuri'!D18</f>
+        <f>'Lista de prețuri'!D16</f>
         <v/>
       </c>
       <c r="E12">
-        <f>IF(ISNUMBER('Lista de prețuri'!E18),'Lista de prețuri'!E18,"")</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E16),'Lista de prețuri'!E16,"")</f>
         <v/>
       </c>
       <c r="F12" t="inlineStr">
@@ -4511,7 +4512,7 @@
     </row>
     <row r="13">
       <c r="A13">
-        <f>'Lista de prețuri'!C19</f>
+        <f>'Lista de prețuri'!C17</f>
         <v/>
       </c>
       <c r="B13" t="inlineStr">
@@ -4520,15 +4521,15 @@
         </is>
       </c>
       <c r="C13">
-        <f>IF(ISNUMBER('Lista de prețuri'!E19),'Lista de prețuri'!E19,IF(ISNUMBER('Lista de prețuri'!D19),'Lista de prețuri'!D19,"La cerere"))</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E17),'Lista de prețuri'!E17,IF(ISNUMBER('Lista de prețuri'!D17),'Lista de prețuri'!D17,"La cerere"))</f>
         <v/>
       </c>
       <c r="D13">
-        <f>'Lista de prețuri'!D19</f>
+        <f>'Lista de prețuri'!D17</f>
         <v/>
       </c>
       <c r="E13">
-        <f>IF(ISNUMBER('Lista de prețuri'!E19),'Lista de prețuri'!E19,"")</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E17),'Lista de prețuri'!E17,"")</f>
         <v/>
       </c>
       <c r="F13" t="inlineStr">
@@ -4544,7 +4545,7 @@
     </row>
     <row r="14">
       <c r="A14">
-        <f>'Lista de prețuri'!C20</f>
+        <f>'Lista de prețuri'!C18</f>
         <v/>
       </c>
       <c r="B14" t="inlineStr">
@@ -4553,15 +4554,15 @@
         </is>
       </c>
       <c r="C14">
-        <f>IF(ISNUMBER('Lista de prețuri'!E20),'Lista de prețuri'!E20,IF(ISNUMBER('Lista de prețuri'!D20),'Lista de prețuri'!D20,"La cerere"))</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E18),'Lista de prețuri'!E18,IF(ISNUMBER('Lista de prețuri'!D18),'Lista de prețuri'!D18,"La cerere"))</f>
         <v/>
       </c>
       <c r="D14">
-        <f>'Lista de prețuri'!D20</f>
+        <f>'Lista de prețuri'!D18</f>
         <v/>
       </c>
       <c r="E14">
-        <f>IF(ISNUMBER('Lista de prețuri'!E20),'Lista de prețuri'!E20,"")</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E18),'Lista de prețuri'!E18,"")</f>
         <v/>
       </c>
       <c r="F14" t="inlineStr">
@@ -4577,7 +4578,7 @@
     </row>
     <row r="15">
       <c r="A15">
-        <f>'Lista de prețuri'!C21</f>
+        <f>'Lista de prețuri'!C19</f>
         <v/>
       </c>
       <c r="B15" t="inlineStr">
@@ -4586,15 +4587,15 @@
         </is>
       </c>
       <c r="C15">
-        <f>IF(ISNUMBER('Lista de prețuri'!E21),'Lista de prețuri'!E21,IF(ISNUMBER('Lista de prețuri'!D21),'Lista de prețuri'!D21,"La cerere"))</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E19),'Lista de prețuri'!E19,IF(ISNUMBER('Lista de prețuri'!D19),'Lista de prețuri'!D19,"La cerere"))</f>
         <v/>
       </c>
       <c r="D15">
-        <f>'Lista de prețuri'!D21</f>
+        <f>'Lista de prețuri'!D19</f>
         <v/>
       </c>
       <c r="E15">
-        <f>IF(ISNUMBER('Lista de prețuri'!E21),'Lista de prețuri'!E21,"")</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E19),'Lista de prețuri'!E19,"")</f>
         <v/>
       </c>
       <c r="F15" t="inlineStr">
@@ -4610,7 +4611,7 @@
     </row>
     <row r="16">
       <c r="A16">
-        <f>'Lista de prețuri'!C23</f>
+        <f>'Lista de prețuri'!C21</f>
         <v/>
       </c>
       <c r="B16" t="inlineStr">
@@ -4619,15 +4620,15 @@
         </is>
       </c>
       <c r="C16">
-        <f>IF(ISNUMBER('Lista de prețuri'!E23),'Lista de prețuri'!E23,IF(ISNUMBER('Lista de prețuri'!D23),'Lista de prețuri'!D23,"La cerere"))</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E21),'Lista de prețuri'!E21,IF(ISNUMBER('Lista de prețuri'!D21),'Lista de prețuri'!D21,"La cerere"))</f>
         <v/>
       </c>
       <c r="D16">
-        <f>'Lista de prețuri'!D23</f>
+        <f>'Lista de prețuri'!D21</f>
         <v/>
       </c>
       <c r="E16">
-        <f>IF(ISNUMBER('Lista de prețuri'!E23),'Lista de prețuri'!E23,"")</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E21),'Lista de prețuri'!E21,"")</f>
         <v/>
       </c>
       <c r="F16" t="inlineStr">
@@ -4643,7 +4644,7 @@
     </row>
     <row r="17">
       <c r="A17">
-        <f>'Lista de prețuri'!C24</f>
+        <f>'Lista de prețuri'!C22</f>
         <v/>
       </c>
       <c r="B17" t="inlineStr">
@@ -4652,15 +4653,15 @@
         </is>
       </c>
       <c r="C17">
-        <f>IF(ISNUMBER('Lista de prețuri'!E24),'Lista de prețuri'!E24,IF(ISNUMBER('Lista de prețuri'!D24),'Lista de prețuri'!D24,"La cerere"))</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E22),'Lista de prețuri'!E22,IF(ISNUMBER('Lista de prețuri'!D22),'Lista de prețuri'!D22,"La cerere"))</f>
         <v/>
       </c>
       <c r="D17">
-        <f>'Lista de prețuri'!D24</f>
+        <f>'Lista de prețuri'!D22</f>
         <v/>
       </c>
       <c r="E17">
-        <f>IF(ISNUMBER('Lista de prețuri'!E24),'Lista de prețuri'!E24,"")</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E22),'Lista de prețuri'!E22,"")</f>
         <v/>
       </c>
       <c r="F17" t="inlineStr">
@@ -4676,7 +4677,7 @@
     </row>
     <row r="18">
       <c r="A18">
-        <f>'Lista de prețuri'!C25</f>
+        <f>'Lista de prețuri'!C23</f>
         <v/>
       </c>
       <c r="B18" t="inlineStr">
@@ -4685,15 +4686,15 @@
         </is>
       </c>
       <c r="C18">
-        <f>IF(ISNUMBER('Lista de prețuri'!E25),'Lista de prețuri'!E25,IF(ISNUMBER('Lista de prețuri'!D25),'Lista de prețuri'!D25,"La cerere"))</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E23),'Lista de prețuri'!E23,IF(ISNUMBER('Lista de prețuri'!D23),'Lista de prețuri'!D23,"La cerere"))</f>
         <v/>
       </c>
       <c r="D18">
-        <f>'Lista de prețuri'!D25</f>
+        <f>'Lista de prețuri'!D23</f>
         <v/>
       </c>
       <c r="E18">
-        <f>IF(ISNUMBER('Lista de prețuri'!E25),'Lista de prețuri'!E25,"")</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E23),'Lista de prețuri'!E23,"")</f>
         <v/>
       </c>
       <c r="F18" t="inlineStr">
@@ -4709,7 +4710,7 @@
     </row>
     <row r="19">
       <c r="A19">
-        <f>'Lista de prețuri'!C26</f>
+        <f>'Lista de prețuri'!C24</f>
         <v/>
       </c>
       <c r="B19" t="inlineStr">
@@ -4718,15 +4719,15 @@
         </is>
       </c>
       <c r="C19">
-        <f>IF(ISNUMBER('Lista de prețuri'!E26),'Lista de prețuri'!E26,IF(ISNUMBER('Lista de prețuri'!D26),'Lista de prețuri'!D26,"La cerere"))</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E24),'Lista de prețuri'!E24,IF(ISNUMBER('Lista de prețuri'!D24),'Lista de prețuri'!D24,"La cerere"))</f>
         <v/>
       </c>
       <c r="D19">
-        <f>'Lista de prețuri'!D26</f>
+        <f>'Lista de prețuri'!D24</f>
         <v/>
       </c>
       <c r="E19">
-        <f>IF(ISNUMBER('Lista de prețuri'!E26),'Lista de prețuri'!E26,"")</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E24),'Lista de prețuri'!E24,"")</f>
         <v/>
       </c>
       <c r="F19" t="inlineStr">
@@ -4742,7 +4743,7 @@
     </row>
     <row r="20">
       <c r="A20">
-        <f>'Lista de prețuri'!C27</f>
+        <f>'Lista de prețuri'!C25</f>
         <v/>
       </c>
       <c r="B20" t="inlineStr">
@@ -4751,15 +4752,15 @@
         </is>
       </c>
       <c r="C20">
-        <f>IF(ISNUMBER('Lista de prețuri'!E27),'Lista de prețuri'!E27,IF(ISNUMBER('Lista de prețuri'!D27),'Lista de prețuri'!D27,"La cerere"))</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E25),'Lista de prețuri'!E25,IF(ISNUMBER('Lista de prețuri'!D25),'Lista de prețuri'!D25,"La cerere"))</f>
         <v/>
       </c>
       <c r="D20">
-        <f>'Lista de prețuri'!D27</f>
+        <f>'Lista de prețuri'!D25</f>
         <v/>
       </c>
       <c r="E20">
-        <f>IF(ISNUMBER('Lista de prețuri'!E27),'Lista de prețuri'!E27,"")</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E25),'Lista de prețuri'!E25,"")</f>
         <v/>
       </c>
       <c r="F20" t="inlineStr">
@@ -4775,7 +4776,7 @@
     </row>
     <row r="21">
       <c r="A21">
-        <f>'Lista de prețuri'!C28</f>
+        <f>'Lista de prețuri'!C26</f>
         <v/>
       </c>
       <c r="B21" t="inlineStr">
@@ -4784,15 +4785,15 @@
         </is>
       </c>
       <c r="C21">
-        <f>IF(ISNUMBER('Lista de prețuri'!E28),'Lista de prețuri'!E28,IF(ISNUMBER('Lista de prețuri'!D28),'Lista de prețuri'!D28,"La cerere"))</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E26),'Lista de prețuri'!E26,IF(ISNUMBER('Lista de prețuri'!D26),'Lista de prețuri'!D26,"La cerere"))</f>
         <v/>
       </c>
       <c r="D21">
-        <f>'Lista de prețuri'!D28</f>
+        <f>'Lista de prețuri'!D26</f>
         <v/>
       </c>
       <c r="E21">
-        <f>IF(ISNUMBER('Lista de prețuri'!E28),'Lista de prețuri'!E28,"")</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E26),'Lista de prețuri'!E26,"")</f>
         <v/>
       </c>
       <c r="F21" t="inlineStr">
@@ -4808,7 +4809,7 @@
     </row>
     <row r="22">
       <c r="A22">
-        <f>'Lista de prețuri'!C29</f>
+        <f>'Lista de prețuri'!C27</f>
         <v/>
       </c>
       <c r="B22" t="inlineStr">
@@ -4817,15 +4818,15 @@
         </is>
       </c>
       <c r="C22">
-        <f>IF(ISNUMBER('Lista de prețuri'!E29),'Lista de prețuri'!E29,IF(ISNUMBER('Lista de prețuri'!D29),'Lista de prețuri'!D29,"La cerere"))</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E27),'Lista de prețuri'!E27,IF(ISNUMBER('Lista de prețuri'!D27),'Lista de prețuri'!D27,"La cerere"))</f>
         <v/>
       </c>
       <c r="D22">
-        <f>'Lista de prețuri'!D29</f>
+        <f>'Lista de prețuri'!D27</f>
         <v/>
       </c>
       <c r="E22">
-        <f>IF(ISNUMBER('Lista de prețuri'!E29),'Lista de prețuri'!E29,"")</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E27),'Lista de prețuri'!E27,"")</f>
         <v/>
       </c>
       <c r="F22" t="inlineStr">
@@ -4841,7 +4842,7 @@
     </row>
     <row r="23">
       <c r="A23">
-        <f>'Lista de prețuri'!C30</f>
+        <f>'Lista de prețuri'!C28</f>
         <v/>
       </c>
       <c r="B23" t="inlineStr">
@@ -4850,15 +4851,15 @@
         </is>
       </c>
       <c r="C23">
-        <f>IF(ISNUMBER('Lista de prețuri'!E30),'Lista de prețuri'!E30,IF(ISNUMBER('Lista de prețuri'!D30),'Lista de prețuri'!D30,"La cerere"))</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E28),'Lista de prețuri'!E28,IF(ISNUMBER('Lista de prețuri'!D28),'Lista de prețuri'!D28,"La cerere"))</f>
         <v/>
       </c>
       <c r="D23">
-        <f>'Lista de prețuri'!D30</f>
+        <f>'Lista de prețuri'!D28</f>
         <v/>
       </c>
       <c r="E23">
-        <f>IF(ISNUMBER('Lista de prețuri'!E30),'Lista de prețuri'!E30,"")</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E28),'Lista de prețuri'!E28,"")</f>
         <v/>
       </c>
       <c r="F23" t="inlineStr">
@@ -4874,19 +4875,19 @@
     </row>
     <row r="24">
       <c r="A24">
-        <f>'Lista de prețuri'!C32</f>
+        <f>'Lista de prețuri'!C30</f>
         <v/>
       </c>
       <c r="C24">
-        <f>IF(ISNUMBER('Lista de prețuri'!E32),'Lista de prețuri'!E32,IF(ISNUMBER('Lista de prețuri'!D32),'Lista de prețuri'!D32,"La cerere"))</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E30),'Lista de prețuri'!E30,IF(ISNUMBER('Lista de prețuri'!D30),'Lista de prețuri'!D30,"La cerere"))</f>
         <v/>
       </c>
       <c r="D24">
-        <f>'Lista de prețuri'!D32</f>
+        <f>'Lista de prețuri'!D30</f>
         <v/>
       </c>
       <c r="E24">
-        <f>IF(ISNUMBER('Lista de prețuri'!E32),'Lista de prețuri'!E32,"")</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E30),'Lista de prețuri'!E30,"")</f>
         <v/>
       </c>
       <c r="F24" t="inlineStr">
@@ -4902,19 +4903,19 @@
     </row>
     <row r="25">
       <c r="A25">
-        <f>'Lista de prețuri'!C33</f>
+        <f>'Lista de prețuri'!C31</f>
         <v/>
       </c>
       <c r="C25">
-        <f>IF(ISNUMBER('Lista de prețuri'!E33),'Lista de prețuri'!E33,IF(ISNUMBER('Lista de prețuri'!D33),'Lista de prețuri'!D33,"La cerere"))</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E31),'Lista de prețuri'!E31,IF(ISNUMBER('Lista de prețuri'!D31),'Lista de prețuri'!D31,"La cerere"))</f>
         <v/>
       </c>
       <c r="D25">
-        <f>'Lista de prețuri'!D33</f>
+        <f>'Lista de prețuri'!D31</f>
         <v/>
       </c>
       <c r="E25">
-        <f>IF(ISNUMBER('Lista de prețuri'!E33),'Lista de prețuri'!E33,"")</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E31),'Lista de prețuri'!E31,"")</f>
         <v/>
       </c>
       <c r="F25" t="inlineStr">
@@ -4930,7 +4931,7 @@
     </row>
     <row r="26">
       <c r="A26">
-        <f>'Lista de prețuri'!C34</f>
+        <f>'Lista de prețuri'!C32</f>
         <v/>
       </c>
       <c r="B26" t="inlineStr">
@@ -4939,15 +4940,15 @@
         </is>
       </c>
       <c r="C26">
-        <f>IF(ISNUMBER('Lista de prețuri'!E34),'Lista de prețuri'!E34,IF(ISNUMBER('Lista de prețuri'!D34),'Lista de prețuri'!D34,"La cerere"))</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E32),'Lista de prețuri'!E32,IF(ISNUMBER('Lista de prețuri'!D32),'Lista de prețuri'!D32,"La cerere"))</f>
         <v/>
       </c>
       <c r="D26">
-        <f>'Lista de prețuri'!D34</f>
+        <f>'Lista de prețuri'!D32</f>
         <v/>
       </c>
       <c r="E26">
-        <f>IF(ISNUMBER('Lista de prețuri'!E34),'Lista de prețuri'!E34,"")</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E32),'Lista de prețuri'!E32,"")</f>
         <v/>
       </c>
       <c r="F26" t="inlineStr">
@@ -4963,7 +4964,7 @@
     </row>
     <row r="27">
       <c r="A27">
-        <f>'Lista de prețuri'!C36</f>
+        <f>'Lista de prețuri'!C34</f>
         <v/>
       </c>
       <c r="B27" t="inlineStr">
@@ -4972,15 +4973,15 @@
         </is>
       </c>
       <c r="C27">
-        <f>IF(ISNUMBER('Lista de prețuri'!E36),'Lista de prețuri'!E36,IF(ISNUMBER('Lista de prețuri'!D36),'Lista de prețuri'!D36,"La cerere"))</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E34),'Lista de prețuri'!E34,IF(ISNUMBER('Lista de prețuri'!D34),'Lista de prețuri'!D34,"La cerere"))</f>
         <v/>
       </c>
       <c r="D27">
-        <f>'Lista de prețuri'!D36</f>
+        <f>'Lista de prețuri'!D34</f>
         <v/>
       </c>
       <c r="E27">
-        <f>IF(ISNUMBER('Lista de prețuri'!E36),'Lista de prețuri'!E36,"")</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E34),'Lista de prețuri'!E34,"")</f>
         <v/>
       </c>
       <c r="F27" t="inlineStr">
@@ -4996,7 +4997,7 @@
     </row>
     <row r="28">
       <c r="A28">
-        <f>'Lista de prețuri'!C37</f>
+        <f>'Lista de prețuri'!C35</f>
         <v/>
       </c>
       <c r="B28" t="inlineStr">
@@ -5005,15 +5006,15 @@
         </is>
       </c>
       <c r="C28">
-        <f>IF(ISNUMBER('Lista de prețuri'!E37),'Lista de prețuri'!E37,IF(ISNUMBER('Lista de prețuri'!D37),'Lista de prețuri'!D37,"La cerere"))</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E35),'Lista de prețuri'!E35,IF(ISNUMBER('Lista de prețuri'!D35),'Lista de prețuri'!D35,"La cerere"))</f>
         <v/>
       </c>
       <c r="D28">
-        <f>'Lista de prețuri'!D37</f>
+        <f>'Lista de prețuri'!D35</f>
         <v/>
       </c>
       <c r="E28">
-        <f>IF(ISNUMBER('Lista de prețuri'!E37),'Lista de prețuri'!E37,"")</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E35),'Lista de prețuri'!E35,"")</f>
         <v/>
       </c>
       <c r="F28" t="inlineStr">
@@ -5029,7 +5030,7 @@
     </row>
     <row r="29">
       <c r="A29">
-        <f>'Lista de prețuri'!C38</f>
+        <f>'Lista de prețuri'!C36</f>
         <v/>
       </c>
       <c r="B29" t="inlineStr">
@@ -5038,15 +5039,15 @@
         </is>
       </c>
       <c r="C29">
-        <f>IF(ISNUMBER('Lista de prețuri'!E38),'Lista de prețuri'!E38,IF(ISNUMBER('Lista de prețuri'!D38),'Lista de prețuri'!D38,"La cerere"))</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E36),'Lista de prețuri'!E36,IF(ISNUMBER('Lista de prețuri'!D36),'Lista de prețuri'!D36,"La cerere"))</f>
         <v/>
       </c>
       <c r="D29">
-        <f>'Lista de prețuri'!D38</f>
+        <f>'Lista de prețuri'!D36</f>
         <v/>
       </c>
       <c r="E29">
-        <f>IF(ISNUMBER('Lista de prețuri'!E38),'Lista de prețuri'!E38,"")</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E36),'Lista de prețuri'!E36,"")</f>
         <v/>
       </c>
       <c r="F29" t="inlineStr">
@@ -5062,7 +5063,7 @@
     </row>
     <row r="30">
       <c r="A30">
-        <f>'Lista de prețuri'!C39</f>
+        <f>'Lista de prețuri'!C37</f>
         <v/>
       </c>
       <c r="B30" t="inlineStr">
@@ -5071,15 +5072,15 @@
         </is>
       </c>
       <c r="C30">
-        <f>IF(ISNUMBER('Lista de prețuri'!E39),'Lista de prețuri'!E39,IF(ISNUMBER('Lista de prețuri'!D39),'Lista de prețuri'!D39,"La cerere"))</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E37),'Lista de prețuri'!E37,IF(ISNUMBER('Lista de prețuri'!D37),'Lista de prețuri'!D37,"La cerere"))</f>
         <v/>
       </c>
       <c r="D30">
-        <f>'Lista de prețuri'!D39</f>
+        <f>'Lista de prețuri'!D37</f>
         <v/>
       </c>
       <c r="E30">
-        <f>IF(ISNUMBER('Lista de prețuri'!E39),'Lista de prețuri'!E39,"")</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E37),'Lista de prețuri'!E37,"")</f>
         <v/>
       </c>
       <c r="F30" t="inlineStr">
@@ -5095,7 +5096,7 @@
     </row>
     <row r="31">
       <c r="A31">
-        <f>'Lista de prețuri'!C40</f>
+        <f>'Lista de prețuri'!C38</f>
         <v/>
       </c>
       <c r="B31" t="inlineStr">
@@ -5104,15 +5105,15 @@
         </is>
       </c>
       <c r="C31">
-        <f>IF(ISNUMBER('Lista de prețuri'!E40),'Lista de prețuri'!E40,IF(ISNUMBER('Lista de prețuri'!D40),'Lista de prețuri'!D40,"La cerere"))</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E38),'Lista de prețuri'!E38,IF(ISNUMBER('Lista de prețuri'!D38),'Lista de prețuri'!D38,"La cerere"))</f>
         <v/>
       </c>
       <c r="D31">
-        <f>'Lista de prețuri'!D40</f>
+        <f>'Lista de prețuri'!D38</f>
         <v/>
       </c>
       <c r="E31">
-        <f>IF(ISNUMBER('Lista de prețuri'!E40),'Lista de prețuri'!E40,"")</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E38),'Lista de prețuri'!E38,"")</f>
         <v/>
       </c>
       <c r="F31" t="inlineStr">
@@ -5128,7 +5129,7 @@
     </row>
     <row r="32">
       <c r="A32">
-        <f>'Lista de prețuri'!C41</f>
+        <f>'Lista de prețuri'!C39</f>
         <v/>
       </c>
       <c r="B32" t="inlineStr">
@@ -5137,15 +5138,15 @@
         </is>
       </c>
       <c r="C32">
-        <f>IF(ISNUMBER('Lista de prețuri'!E41),'Lista de prețuri'!E41,IF(ISNUMBER('Lista de prețuri'!D41),'Lista de prețuri'!D41,"La cerere"))</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E39),'Lista de prețuri'!E39,IF(ISNUMBER('Lista de prețuri'!D39),'Lista de prețuri'!D39,"La cerere"))</f>
         <v/>
       </c>
       <c r="D32">
-        <f>'Lista de prețuri'!D41</f>
+        <f>'Lista de prețuri'!D39</f>
         <v/>
       </c>
       <c r="E32">
-        <f>IF(ISNUMBER('Lista de prețuri'!E41),'Lista de prețuri'!E41,"")</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E39),'Lista de prețuri'!E39,"")</f>
         <v/>
       </c>
       <c r="F32" t="inlineStr">
@@ -5161,7 +5162,7 @@
     </row>
     <row r="33">
       <c r="A33">
-        <f>'Lista de prețuri'!C42</f>
+        <f>'Lista de prețuri'!C40</f>
         <v/>
       </c>
       <c r="B33" t="inlineStr">
@@ -5170,15 +5171,15 @@
         </is>
       </c>
       <c r="C33">
-        <f>IF(ISNUMBER('Lista de prețuri'!E42),'Lista de prețuri'!E42,IF(ISNUMBER('Lista de prețuri'!D42),'Lista de prețuri'!D42,"La cerere"))</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E40),'Lista de prețuri'!E40,IF(ISNUMBER('Lista de prețuri'!D40),'Lista de prețuri'!D40,"La cerere"))</f>
         <v/>
       </c>
       <c r="D33">
-        <f>'Lista de prețuri'!D42</f>
+        <f>'Lista de prețuri'!D40</f>
         <v/>
       </c>
       <c r="E33">
-        <f>IF(ISNUMBER('Lista de prețuri'!E42),'Lista de prețuri'!E42,"")</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E40),'Lista de prețuri'!E40,"")</f>
         <v/>
       </c>
       <c r="F33" t="inlineStr">
@@ -5194,7 +5195,7 @@
     </row>
     <row r="34">
       <c r="A34">
-        <f>'Lista de prețuri'!C43</f>
+        <f>'Lista de prețuri'!C41</f>
         <v/>
       </c>
       <c r="B34" t="inlineStr">
@@ -5203,15 +5204,15 @@
         </is>
       </c>
       <c r="C34">
-        <f>IF(ISNUMBER('Lista de prețuri'!E43),'Lista de prețuri'!E43,IF(ISNUMBER('Lista de prețuri'!D43),'Lista de prețuri'!D43,"La cerere"))</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E41),'Lista de prețuri'!E41,IF(ISNUMBER('Lista de prețuri'!D41),'Lista de prețuri'!D41,"La cerere"))</f>
         <v/>
       </c>
       <c r="D34">
-        <f>'Lista de prețuri'!D43</f>
+        <f>'Lista de prețuri'!D41</f>
         <v/>
       </c>
       <c r="E34">
-        <f>IF(ISNUMBER('Lista de prețuri'!E43),'Lista de prețuri'!E43,"")</f>
+        <f>IF(ISNUMBER('Lista de prețuri'!E41),'Lista de prețuri'!E41,"")</f>
         <v/>
       </c>
       <c r="F34" t="inlineStr">

</xml_diff>